<commit_message>
Add trade RFQ leads tab, marketplace costs and safer terms to the RFQ kit
- prospects-minyala.xlsx: new "Demandes RFQ" tab with 52 buyer requests
  (StoneAdd, Alibaba, go4WorldBusiness, TradeKey re-checked on public
  pages; StoneContact ones from search results, marked unverified as the
  site blocks automated access), with reply status tracking. Five trade
  marketplaces added to "Plateformes pros" (Destockplus, StoneAdd,
  StoneContact, Europages, go4WorldBusiness).
- rfq-kit.md: what replying costs on each marketplace, requests to answer
  first, Minya trade names to use only if the origin is confirmed, FCA for
  export, and more fraud rules (MT103 is not payment, paid samples, booby-
  trapped RFQ attachments), with sources.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Xqm9tFtdvLdJdkiWw2VVp6
</commit_message>
<xml_diff>
--- a/minyala/prospects-minyala.xlsx
+++ b/minyala/prospects-minyala.xlsx
@@ -11,11 +11,13 @@
     <sheet name="Mode d'emploi" sheetId="1" state="visible" r:id="rId3"/>
     <sheet name="Prospects" sheetId="2" state="visible" r:id="rId4"/>
     <sheet name="Particuliers" sheetId="3" state="visible" r:id="rId5"/>
-    <sheet name="Groupes Facebook" sheetId="4" state="visible" r:id="rId6"/>
-    <sheet name="Plateformes pros" sheetId="5" state="visible" r:id="rId7"/>
-    <sheet name="Règles" sheetId="6" state="visible" r:id="rId8"/>
+    <sheet name="Demandes RFQ" sheetId="4" state="visible" r:id="rId6"/>
+    <sheet name="Groupes Facebook" sheetId="5" state="visible" r:id="rId7"/>
+    <sheet name="Plateformes pros" sheetId="6" state="visible" r:id="rId8"/>
+    <sheet name="Règles" sheetId="7" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames>
+    <definedName function="false" hidden="true" localSheetId="3" name="_xlnm._FilterDatabase" vbProcedure="false">'Demandes RFQ'!$A$1:$N$53</definedName>
     <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">Prospects!$A$1:$Q$198</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
@@ -76,7 +78,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2499" uniqueCount="1269">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3140" uniqueCount="1616">
   <si>
     <t xml:space="preserve">Prospection MINYALA — mode d'emploi</t>
   </si>
@@ -93,7 +95,7 @@
     <t xml:space="preserve">4. Particuliers : pas de liste de personnes (interdit sans leur accord). L'onglet Particuliers liste où les trouver : annonces, forums, foires, publicité.</t>
   </si>
   <si>
-    <t xml:space="preserve">5. Onglet Groupes Facebook : groupes repérés, à approcher avec l'accord des administrateurs (jamais d'extraction de membres). Onglet Règles : ce qui est autorisé pour appeler, écrire ou publier. Important : on ne peut plus appeler un particulier sans son accord.</t>
+    <t xml:space="preserve">5. Onglet Demandes RFQ : demandes d'acheteurs pros repérées sur StoneContact, StoneAdd, Alibaba, go4WorldBusiness, TradeKey (répondre depuis votre compte). Onglet Groupes Facebook : groupes repérés, à approcher avec l'accord des administrateurs (jamais d'extraction de membres). Onglet Règles : ce qui est autorisé pour appeler, écrire ou publier. Important : on ne peut plus appeler un particulier sans son accord.</t>
   </si>
   <si>
     <t xml:space="preserve">Les entreprises ont été vérifiées sur leur site ou un annuaire en ligne (08/10 et 12/10/2026). Vérifiez avant de vous déplacer.</t>
@@ -3387,6 +3389,993 @@
     <t xml:space="preserve">• À décider : échantillons à retirer à Gennevilliers, tarif pour poseurs partenaires. Rien de cela n'existe aujourd'hui sur le site.</t>
   </si>
   <si>
+    <t xml:space="preserve">Correspondance</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vérifiée ?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Plateforme</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Demande</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Produit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Quantité</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Format</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Destination</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Date</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pourquoi / attention</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Répondu le</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forte</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Oui</t>
+  </si>
+  <si>
+    <t xml:space="preserve">StoneAdd</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Buy Sunny Marble</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sunny Marble (catégorie « Egypt Marbles »), donc la pierre calcaire Sunny de Minya</t>
+  </si>
+  <si>
+    <t xml:space="preserve">non précisée</t>
+  </si>
+  <si>
+    <t xml:space="preserve">non précisé</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Autriche (livraisons Autriche et sud de l'Allemagne)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-05-19</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pierre égyptienne Sunny, de la même famille que la Minyala (Minya). L'acheteur est un grossiste qui livre toute l'Autriche et le sud de l'Allemagne, ce qui en fait un débouché européen proche. Il demande si la pierre résiste au gel.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">À étudier</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ataija Creme Limestone Inquiry</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Calcaire crème Ataija (Portugal) pour terrasse et piscine</t>
+  </si>
+  <si>
+    <t xml:space="preserve">100 m²</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Belgique</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-08-17</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Demande de calcaire crème en petite quantité (100 m²) depuis la Belgique, à distance de camion de Gennevilliers. La Minyala peut être proposée comme alternative beige. Attention : l'usage est extérieur (piscine), il faut donc vérifier la résistance au gel et l'antidérapant.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alibaba RFQ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Perfekte Steinfliesen aus Kalkstein und Marmor für Innenräume, Natürliche Kalksteinplatten für Hausrenovierung und Wohnprojekte</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Carreaux de sol en pierre naturelle (calcaire ou marbre) pour l'intérieur et la rénovation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">40 pièces (MOQ en m² demandé)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Suisse</t>
+  </si>
+  <si>
+    <t xml:space="preserve">affiché « 10 days ago » le 2026-10-12 (vers le 2026-10-02)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Carreaux de calcaire pour sol intérieur, acheteur en Suisse, pays voisin de la France. Il demande un catalogue et un MOQ en m², ce qui correspond à une vente sur stock à partir de 25 m². Pour répondre sur Alibaba, il faut un abonnement vendeur payant.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Non (StoneContact bloqué)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">StoneContact</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Beaumaniere Limestone Slabs &amp; Tiles, France Beige Limestone from France (buyer request on the listing)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Unpolished limestone tile, warm beige, grey or brown, not too light (Beaumaniere given as the reference)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">about 150 m²</t>
+  </si>
+  <si>
+    <t xml:space="preserve">at least 60x30 or 60x40 cm, unpolished</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rotterdam, Netherlands</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Calcaire beige non poli, format minimum 60x30, 150 m², destination Pays-Bas (Rotterdam) : correspond très bien à MINYALA 30x60 en stock. Mais la demande n'est pas datée et est probablement ancienne.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sinai Pearl Grey Limestone Slabs&amp;Tiles from Egypt</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sinai Pearl Grey limestone (Egyptian) tiles, with a sample requested before ordering</t>
+  </si>
+  <si>
+    <t xml:space="preserve">150 m²</t>
+  </si>
+  <si>
+    <t xml:space="preserve">France (clients in France and the UK)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Entreprise française de rénovation qui cherche du calcaire égyptien pour des clients en France et au Royaume-Uni, 150 m², échantillon d'abord : le stock de Gennevilliers permet un échantillon et une livraison rapides. La teinte demandée est grise et non crème, et la demande n'est pas datée.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Possible</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Marble Slabs Inquiry</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tranches de marbre, environ 150 m², achat sur stock</t>
+  </si>
+  <si>
+    <t xml:space="preserve">environ 150 m²</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-07-15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L'acheteur est en France et veut environ 150 m² disponibles en stock, avec visite sur place. Un stock à Gennevilliers convient très bien sur la logistique. En revanche, il cherche du « marbre » en tranches et non des carreaux 30×60 : à proposer comme alternative.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">go4WorldBusiness</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Wanted : Marble</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Marbre blanc ou crème, dimensions sur mesure</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 conteneur 20'</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sur mesure</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Espagne</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-07-09</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Acheteur espagnol qui cherche du marbre crème et préfère un fournisseur européen, ce qui avantage un vendeur basé en France. Le volume (1 conteneur 20') dépasse sans doute le stock, et le paiement se fait FOB par virement.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Wanted : Stone Articles Like Marble, Granite, Limestone</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Articles en pierre (marbre, granit, calcaire, ardoise) pour la construction et la revente (HS 680299)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-09-29</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Acheteur en France qui inclut le calcaire, pour la revente et la distribution. Le produit reste vague (articles décoratifs) et porte sur 1 conteneur 20'. La proximité est un atout.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Wanted : Natural Stones Like Sandstone, Limestone</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Grès, calcaire et mosaïques de pierre naturelle, tailles sur mesure</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Allemagne</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-06-26</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Acheteur allemand qui inclut le calcaire en tailles sur mesure. La quantité (1 conteneur 20') et la couleur ne sont pas précisées. L'annonce, du 26 juin, approche de sa date d'expiration.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Buy Crema Marfil tiles 305x305x1cm Standard Range</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Carreaux de marbre beige Crema Marfil 30,5×30,5×1 cm, polis</t>
+  </si>
+  <si>
+    <t xml:space="preserve">30,5×30,5×1 cm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-04-18</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Carreaux de marbre beige demandés depuis l'Espagne, avec une question sur le stock. Le format (30,5×30,5×1 cm) et la pierre (espagnole) ne sont pas les mêmes que la Minyala 30×60×2. À proposer comme alternative moins chère. La demande date d'avril.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Buy Moscato Beige Marble</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Marbre beige Moscato (Espagne)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Irlande</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-09-12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pierre beige, acheteur en Irlande (UE). La demande vise une référence espagnole précise et ne donne ni format ni quantité.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Buy THALA BEIGE Marbles</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Thala Beige (pierre beige tunisienne)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Italie</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-08-29</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pierre beige nord-africaine du même registre que la Minyala, acheteur en Italie. La demande est générique et sans quantité.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Buy Sinai Pearl Limestone Stairs and Steps</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Marches et escaliers en calcaire égyptien Sinai Pearl</t>
+  </si>
+  <si>
+    <t xml:space="preserve">marches (non précisé)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kosovo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-09-09</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Calcaire égyptien, acheteur au Kosovo (Europe hors UE). Il cherche des marches et non des carreaux 30×60, et la Sinai Pearl vient du Sinaï, pas de Minya.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Buy Turkey Ivory Travertine Slab</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Travertin ivoire (Turquie), 120 m², livraison à Kalamata</t>
+  </si>
+  <si>
+    <t xml:space="preserve">120 m²</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kalamata, Grèce</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-06-05</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pierre claire en petite quantité (120 m²) pour la Grèce, dans l'UE. C'est du travertin et non du calcaire, et le transport jusqu'à Kalamata coûte cher depuis Paris.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Beige Travertine KARAMAN Inquiry</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Travertin beige de Karaman : dalles 1,2×40,6×61, margelles 3×33×61 et angles 3×48×48</t>
+  </si>
+  <si>
+    <t xml:space="preserve">non précisée (importateur d'environ 40 conteneurs par an)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1,2×40,6×61 cm ; 3×33×61 cm ; 3×48×48 cm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">France (Sud-Ouest)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-03-27</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Importateur français de pierre beige installé dans le Sud-Ouest (environ 40 conteneurs par an), insatisfait de ses fournisseurs actuels. C'est un bon prospect commercial, mais il demande du travertin turc dans des formats précis, pas du calcaire 30×60.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Galala Extra - Galala Marble Quarry</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Commercial-grade Galala Extra (Egyptian beige), bush-hammered top face, other faces sawn</t>
+  </si>
+  <si>
+    <t xml:space="preserve">about 3,950 m² in total (2,570 m² of it in 60x30)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">60x30x7.5, 60x25x7.5, 30x30x7.5, 100x30x7.5, 100x50x7.5 cm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">France (French project)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pierre beige égyptienne pour un projet en France avec un gros volume en 60x30, mais l'épaisseur demandée est de 7,5 cm (dallage), contre 2 cm pour MINYALA. Demande non datée.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sinai Pearl Limestone Tiles &amp; Slabs, Grey Limestone Egypt Polished Floor Covering Tiles, Walling Tiles from Egypt</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Honed Sinai Pearl limestone tiles</t>
+  </si>
+  <si>
+    <t xml:space="preserve">30 m²</t>
+  </si>
+  <si>
+    <t xml:space="preserve">600x400x15 mm, honed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cardiff, Wales, UK</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Petit volume (30 m², au-dessus du minimum de 25 m²) de calcaire égyptien adouci livré au Royaume-Uni : MINYALA peut proposer le 30x60x2 comme alternative au 60x40x1,5. Demande non datée.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Buyers from United Kingdom - Global Stone Buyer Center (RFQ for Oman White Limestone)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Oman White limestone, as slabs or cut-to-size tiles</t>
+  </si>
+  <si>
+    <t xml:space="preserve">65 m²</t>
+  </si>
+  <si>
+    <t xml:space="preserve">slabs or cut-to-size, 20 mm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">London, UK</t>
+  </si>
+  <si>
+    <t xml:space="preserve">May 14, 2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Demande récente (mai 2026), 65 m² en 20 mm livrés à Londres : volume et épaisseur conviennent. La couleur demandée est blanche (Oman White), pas crème, donc MINYALA ne peut être proposé qu'en alternative.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Westhill Limestone Honed Tiles from United Kingdom</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Honed beige limestone tiles (Westhill), larger formats around 1000x500 also asked about</t>
+  </si>
+  <si>
+    <t xml:space="preserve">about 63 m²</t>
+  </si>
+  <si>
+    <t xml:space="preserve">honed; asks about about 1000x500</t>
+  </si>
+  <si>
+    <t xml:space="preserve">page dated 2025-02-08 (request date not confirmed)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Calcaire beige adouci pour une rénovation à Londres, environ 63 m² : petit volume compatible avec le stock. L'acheteur demande un prix au m² ; il vise une pierre précise et peut-être un grand format.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Beige Limestone Floor Tiles from United Kingdom</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Polished grey-beige Jura limestone</t>
+  </si>
+  <si>
+    <t xml:space="preserve">150 m (as written by the buyer)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">60x40 cm, polished</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Calcaire beige, 150 m² sur une annonce britannique : MINYALA pourrait être proposé en 30x60 à la place du 60x40 Jura poli. Destination non confirmée et demande non datée.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sunny Menia Marble Slabs, Tiles from Egypt</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Slabs and tiles 2-4 cm thick in various formats, 'specially Sinai Pearl or similar' (on a Sunny Menia listing)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2, 3 and 4 cm; various formats</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Barcelona, Spain (CIF)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Acheteur espagnol (CIF Barcelone) intéressé par la pierre beige égyptienne « Sinai Pearl ou similaire » sur une annonce Sunny Menia, donc la famille de MINYALA. Formats variés de 2 à 4 cm ; demande non datée.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Galala Beige Marble Tiles &amp; Slab from Egypt</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Galala (Egyptian beige), 80x80x2 honed tiles filled with epoxy resin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7,000 m²</t>
+  </si>
+  <si>
+    <t xml:space="preserve">80x80x2 cm, honed, epoxy-filled</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Spain (Spanish company)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Projet espagnol de 7 000 m² en pierre beige égyptienne de 2 cm adoucie : la teinte et l'épaisseur conviennent, mais le format 80x80 et le volume dépassent le stock. Demande non datée.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dijon Limestone Honed Finish Floor Tiles from United Kingdom</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dijon beige limestone for exterior paving</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2,000 m²</t>
+  </si>
+  <si>
+    <t xml:space="preserve">60x30, 60x20, 60x15, 40x40 cm; 5 cm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Spain (company located in Spain)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Calcaire beige en 60x30 demandé par une société espagnole d'import-export (2 000 m²), mais pour du dallage extérieur en 5 cm : l'épaisseur ne correspond pas aux 2 cm de MINYALA. Demande non datée.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Global Stone Buyer Center (RFQ for Portuguese Moleanos Beige Limestone)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cut-to-size honed tiles in Moleanos Beige limestone (Portugal)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cut-to-size, honed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Russia</t>
+  </si>
+  <si>
+    <t xml:space="preserve">May 26, 2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Calcaire beige adouci sur mesure, demande récente (mai 2026), mais l'acheteur veut du Moleanos portugais et livraison en Russie (EXW). La substitution par MINYALA est peu probable et le volume (2 000 m²) dépasse le stock.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sinai Pearl Limestone - Tumbled Limestone - Egyptian Limestone Supplier from Egypt</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sinai Pearl limestone tiles (Egyptian)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">100 to 200 m²</t>
+  </si>
+  <si>
+    <t xml:space="preserve">preferably 600x900 mm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Petit volume (100 à 200 m²) de calcaire égyptien, adapté à un stock disponible. Format souhaité 60x90, destination non indiquée, demande non datée.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sinai Pearl Limestone - Beige Limestone</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sinai Pearl limestone (Egyptian), for a trader's client</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4,000 m²</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Négociant qui cherche du calcaire beige égyptien pour un client : piste pour proposer MINYALA en alternative, mais 4 000 m² dépasse probablement le stock. Destination et date non indiquées.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Buyers from France - Global Stone Buyer Center (RFQ for beige sandstone flooring)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Beige sandstone flooring with a natural surface (photos attached)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">about 300 m²</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aug 21, 2025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Acheteur en France, environ 300 m² de dallage beige : MINYALA pourrait être proposé comme alternative calcaire. La demande vise du grès et date d'août 2025, juste au-delà de 12 mois.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Buyers from France - Global Stone Buyer Center (RFQ for Buffon Banc Limestone)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Buffon Banc limestone (French beige limestone); photos and price per m² requested</t>
+  </si>
+  <si>
+    <t xml:space="preserve">July 2025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Acheteur français de calcaire beige : on peut lui proposer MINYALA comme alternative moins chère livrée depuis Gennevilliers. Il vise toutefois une pierre française précise, et la demande date de juillet 2025.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Buyers from Ireland - Global Stone Buyer Center (RFQ for Jerusalem Gold Limestone tiles and cobbles)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jerusalem Gold limestone: sanded exterior slabs, kerbs, tumbled cobbles (landscaping)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">a few hundred metres</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sanded finish</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ireland</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aug 27, 2025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Calcaire doré-beige pour l'extérieur en Irlande, « quelques centaines de mètres » : MINYALA peut être proposé pour les dalles. Il s'agit surtout d'aménagement paysager, et la demande date d'août 2025.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Faible</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Oui (corrigée)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sunny Beige Marble Tiles Quotation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Carreaux de Sunny Beige égyptien en petit format (2×2)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2×2 (pouces)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">États-Unis</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-05-06</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Correction : Size: '2x2' (units not stated on the page; the buyer also asks whether smaller sizes exist). Quantity: not stated. Destination: USA. Date: 2026-05-06. — Le produit est exactement la famille Sunny de Minya, mais l'acheteur est aux États-Unis et veut des mosaïques 2×2 pouces. La destination est lointaine et le format ne correspond pas.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bulk Inquiry - 11000 M2 Beige Marble Slabs 60x120cmx2cm EXW Factory</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Plaques de marbre beige clair/crème 60×120×2 cm pour façade, type Silvia Menia ou Sunny Light</t>
+  </si>
+  <si>
+    <t xml:space="preserve">11 000 m²</t>
+  </si>
+  <si>
+    <t xml:space="preserve">60×120×2 cm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Égypte</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-08-31</t>
+  </si>
+  <si>
+    <t xml:space="preserve">La pierre de référence est de la famille Minya, mais l'acheteur est en Égypte, achète EXW usine et veut 11 000 m² en 60×120. Sans rapport avec un stock de 30×60 à Paris.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DIY Interlock Modern Outdoor Anti-slip Stone Deck Tile Floor Marble Tile Limestone Deck Tile Stone ...</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dalles clipsables en travertin beige 300×300×20 sur base plastique (réf. fournisseur PBST-008)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">155 pièces</t>
+  </si>
+  <si>
+    <t xml:space="preserve">300×300×20 mm (10 mm de pierre et 10 mm de plastique)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Londres, Royaume-Uni</t>
+  </si>
+  <si>
+    <t xml:space="preserve">affiché « 1 days ago » le 2026-10-12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Destination Londres et petite quantité, mais l'acheteur veut un produit précis : des dalles de travertin clipsables sur support plastique, différentes de la Minyala.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">bathroom tiles walls and floors</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Carreaux de salle de bain murs et sols, aspect pierre naturelle chaude et neutre, mat, R10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">26 m²</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Portugal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">affiché « 4 days ago » le 2026-10-12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Correction : Product: full-body porcelain floor tiles with a warm neutral natural-stone look, matt, R10, rectified, with matching wall tiles (not natural stone). Size: 800x800x10 mm. Quantity: 26 m². Destination: Portugal. Date: posted 2026-10-08. — Petite quantité au Portugal, mais la description (R10, chauffage au sol, coupes à 45°) évoque plutôt du grès cérame aspect pierre. Le produit n'est pas précisé.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">YDSTONE Beige Tumbled French Pattern Travertine Tile Limestone for Indoor Outdoor Staircases ...</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dalles extérieures en travertin beige adouci, 30 mm minimum, au moins 300×600</t>
+  </si>
+  <si>
+    <t xml:space="preserve">au moins 300×600, épaisseur 30 mm minimum</t>
+  </si>
+  <si>
+    <t xml:space="preserve">affiché « 5 days ago » le 2026-10-12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Correction : Product: outdoor travertine pavers for wet areas, slip-resistant, honed (not polished). Size: width at least 300 mm, length at least 600 mm, thickness at least 30 mm. Quantity: 150 m². Destination: Perth, Australia (buyer account listed as United States). Date: posted 2026-10-06. — Pierre beige au format 30×60 environ, mais l'acheteur est aux États-Unis et demande une épaisseur de 30 mm minimum, alors que la Minyala fait 20 mm.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TradeKey</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DEMANDE PRIX</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Plaque de marbre 60×70 cm pour une salle d'exposition</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 à 10 plaques, puis prix au m²</t>
+  </si>
+  <si>
+    <t xml:space="preserve">60×70 cm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-09-01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Acheteur en France qui veut un prix livré, mais la quantité est minime (1 à 10 plaques) et le format 60×70 diffère du 30×60. Réponse réservée aux membres payants. Les dates TradeKey semblent rafraîchies.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Floor tiles</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Carreaux de sol (tags : limestone, marble, travertine, slate…)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Royaume-Uni</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-08</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Acheteur au Royaume-Uni, mais la demande se résume à « I want to buy floor tiles ». Aucune spécification, et la réponse est réservée aux membres Premium.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Wanted : Natural Stones Like Sawn And Tumbled Finish</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dalles 500×500×30 sciées et vieillies : travertin beige 640 m², gris foncé 447 m², jaune cristal 521 m²</t>
+  </si>
+  <si>
+    <t xml:space="preserve">640 m² (beige), plus d'autres teintes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">500×500×30 mm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Oman</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-07-21</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pierre beige vieillie, mais l'acheteur est à Oman, loin de l'Europe, et demande du 50×50×3 cm.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Wanted : Natural Stone Like Sandstone, Limestone, Natural Stones</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Grès et calcaire sur mesure, noir, brun ou gris</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Split, Croatie</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-09-03</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Calcaire pour l'Europe (Split, Croatie), mais les couleurs voulues sont sombres (noir, brun, gris) et le paiement se fait par L/C pour 1 conteneur.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Request sample for Limestone Beige Split Face</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Échantillon de parement en calcaire beige éclaté (Bulgarie)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">échantillon</t>
+  </si>
+  <si>
+    <t xml:space="preserve">parement éclaté</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-06-08</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Calcaire beige pour le Royaume-Uni, mais il s'agit d'un parement mural éclaté et seulement d'une demande d'échantillon.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Buyers from France - Global Stone Buyer Center (RFQ for limestone stone veneer)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Glued stone veneer in Anstrude Clair and Massangis Clair limestone</t>
+  </si>
+  <si>
+    <t xml:space="preserve">veneer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">September 2025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Acheteur en France, mais le produit demandé est un placage collé en pierres françaises précises (Anstrude, Massangis), pas du carrelage 30x60.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Buyers from Germany - Global Stone Buyer Center (Inquire About Verona Beige Marble)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Verona Beige marble, regular supply wanted</t>
+  </si>
+  <si>
+    <t xml:space="preserve">regular supply (no quantity stated)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Germany</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jul 23, 2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Importateur allemand qui cherche une pierre beige en approvisionnement régulier : on peut le contacter, mais il demande un marbre précis (Verona Beige, Pakistan), pas du calcaire égyptien.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Buyers from Portugal - Global Stone Buyer Center (RFQ for Victory Beige Marble)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Victory Beige marble slabs, 2 cm, honed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">slabs, 2 cm, honed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Oct 8, 2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Demande très récente (oct. 2026) d'une pierre beige de 2 cm adoucie au Portugal, mais en tranches et en marbre précis : substitution par du carrelage 30x60 peu probable.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Buyers from Italy - Global Stone Buyer Center (Caliza Capri Limestone)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Caliza Capri limestone blocks (about 2 for a trial)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">about 2 blocks for a trial</t>
+  </si>
+  <si>
+    <t xml:space="preserve">blocks</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Italy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aug 4, 2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Acheteur en Italie (août 2026), mais il demande des blocs d'un calcaire précis : sans intérêt pour un stock de carreaux.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[RFQ]Inquire About Galala Marble, Black Granite (Buyers from Bahrain)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Polished Galala marble (Egypt origin): flooring and wall cladding</t>
+  </si>
+  <si>
+    <t xml:space="preserve">600x600x20 mm (floor); 1200x600 and 1500x600 mm (cladding)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bahrain</t>
+  </si>
+  <si>
+    <t xml:space="preserve">July 2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pierre beige égyptienne demandée en juillet 2026, mais destination lointaine (Bahreïn), finition polie et formats 60x60 et 120x60 : peu adapté à un stock en France.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Buyers from Kuwait - Global Stone Buyer Center (Turkish light limestone)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Turkish light limestone, off-white, honed tiles</t>
+  </si>
+  <si>
+    <t xml:space="preserve">about 2,000 m²</t>
+  </si>
+  <si>
+    <t xml:space="preserve">40x80x3 cm, honed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kuwait</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mar 9, 2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Calcaire clair adouci, 2 000 m² (mars 2026), mais destination Koweït, origine turque demandée et épaisseur 3 cm.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Buyers from Kuwait - Global Stone Buyer Center (Kota Beige Limestone)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kota Beige limestone (India) for exterior walls</t>
+  </si>
+  <si>
+    <t xml:space="preserve">60x120x3 cm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">July 2026 (Jul 11, 2026)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Calcaire beige, 100 m², mais destination Koweït, format 60x120x3 et pierre indienne précise.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Buyers from United States - Global Stone Buyer Center (Jura Beige Limestone)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jura Beige limestone, large-format tiles and slabs, leather finish, interior flooring</t>
+  </si>
+  <si>
+    <t xml:space="preserve">about 10,000 sq ft</t>
+  </si>
+  <si>
+    <t xml:space="preserve">24x48 in, 1/2 in, leather finish</t>
+  </si>
+  <si>
+    <t xml:space="preserve">United States</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Calcaire beige chaud pour sol intérieur (juillet 2026), mais destination États-Unis, format 24x48 pouces et grand volume.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Natural Stone Buyers from Qatar (Limra Limestone, villa in Doha)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cut-to-size Limra limestone for a villa exterior</t>
+  </si>
+  <si>
+    <t xml:space="preserve">about 2,288 m²</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cut-to-size</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Doha, Qatar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sep 29, 2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Demande récente (29 sept. 2026) mais destination lointaine (Doha) et calcaire blanc turc (Limra) en dimensions sur mesure.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Buyers from Saudi Arabia - Global Stone Buyer Center (Riyadh Stone or similar beige limestone, facades)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Riyadh Stone or a similar beige limestone for facades</t>
+  </si>
+  <si>
+    <t xml:space="preserve">45,000 m²</t>
+  </si>
+  <si>
+    <t xml:space="preserve">60x30 cm, thickness to be confirmed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Saudi Arabia</t>
+  </si>
+  <si>
+    <t xml:space="preserve">April 2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Calcaire beige en 60x30, mais volume énorme (45 000 m²), destination Arabie saoudite et préférence déclarée pour des fournisseurs saoudiens.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Riyadh Limestone Tile from Saudi Arabia</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Beige Riyadh limestone, bush-hammered</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2,700 m²</t>
+  </si>
+  <si>
+    <t xml:space="preserve">30x60x3 cm, bush-hammered</t>
+  </si>
+  <si>
+    <t xml:space="preserve">about 112 days ago (relative to the index snapshot)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Le format 30x60 correspond, mais il s'agit de pierre saoudienne de 3 cm bouchardée, avec destination probablement au Moyen-Orient.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Global Stone Buyer Center - page 3 (RFQ for beige-cream flamed limestone cladding and paving)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Beige-cream limestone, flamed finish, for cladding and paving (technical data sheets requested)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">20 mm; slabs about 140-180 x 250-300 cm; flamed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Egypt (per a search summary, unconfirmed)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aug 25, 2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">La couleur beige-crème et les 20 mm correspondent, mais la demande porte sur de grandes tranches flammées et des fiches techniques pour un projet. Destination incertaine (Égypte selon un résumé).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sunny Menia Marble - Beige Marble</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sunny Menia (Minya stone), acid-washed / honed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">300x300x18 mm, acid-washed / honed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Shenzhen, China</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Exactement la famille de pierre de MINYALA (Sunny Menia, Minya), mais destination Chine (Shenzhen) et format 30x30x1,8 : sans intérêt pour un stock en France.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• « Vérifiée ? = Oui » : la demande a été retrouvée sur la page publique de la plateforme le 12/10/2026.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• StoneContact bloque les accès automatisés : ses demandes viennent de résultats de recherche et n'ont pas pu être revérifiées. Ouvrez-les une fois connecté ; beaucoup sont anciennes ou sans date.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Les coordonnées des acheteurs sont réservées aux membres connectés ou payants. Aucun nom ni contact d'acheteur n'est enregistré ici.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Liens Alibaba : ils peuvent dépendre de la session ; si un lien ne s'ouvre pas, cherchez le titre dans la liste des RFQ Alibaba.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Avant de répondre : lire l'onglet Règles et la section sécurité de rfq-kit.md (jamais de frais à payer, marchandise remise après paiement reçu).</t>
+  </si>
+  <si>
     <t xml:space="preserve">Groupe</t>
   </si>
   <si>
@@ -3790,6 +4779,60 @@
   </si>
   <si>
     <t xml:space="preserve">Contacter les magasins qui ont un rayon Pavés-Dallages et une salle d'exposition (deux sont déjà dans Prospects : Clamart et Houilles).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Destockplus (déstockage B2B France)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pros qui achètent des lots</t>
+  </si>
+  <si>
+    <t xml:space="preserve">France — annonce gratuite (publiée sous 72 h)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Publier le lot MINYALA (500–2 000 m², 27 €/m² TTC pro, dès 25 m², Gennevilliers et Vernon). Concurrent présent à 27 €/m² avec 160 m² minimum.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">StoneAdd (demandes d'acheteurs pierre)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Importateurs, grossistes, poseurs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">International — 27 000+ demandes publiques</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Inscription gratuite, coordonnées des acheteurs réservées au Premium. Meilleures demandes trouvées ici (Autriche, Belgique, France) : voir onglet Demandes RFQ.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Acheteurs de pierre du monde entier</t>
+  </si>
+  <si>
+    <t xml:space="preserve">International</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Créer le compte gratuit et publier la fiche MINYALA (textes dans rfq-kit.md). Ne payer Diamond (≈ 2 000 $/an, non confirmé) qu'après un mois de mesure.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Europages</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Acheteurs professionnels européens</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Europe — page entreprise</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Créer la page entreprise gratuite ; tester le « Request Hub » fournisseur (essai gratuit annoncé).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Importateurs (souvent par conteneur)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">International — abonnement dès 75 $/mois</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Seulement si StoneAdd et StoneContact ne suffisent pas : plusieurs demandes européennes de calcaire / marbre crème.</t>
   </si>
   <si>
     <t xml:space="preserve">ChatGPT (via Shopify)</t>
@@ -4322,6 +5365,10 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
 </file>
 
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office Theme">
   <a:themeElements>
@@ -15196,6 +16243,2250 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
+  <dimension ref="A1:N59"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="36"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="50"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="28"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="14" t="s">
+        <v>1103</v>
+      </c>
+      <c r="B1" s="14" t="s">
+        <v>1104</v>
+      </c>
+      <c r="C1" s="14" t="s">
+        <v>1105</v>
+      </c>
+      <c r="D1" s="14" t="s">
+        <v>1106</v>
+      </c>
+      <c r="E1" s="14" t="s">
+        <v>1107</v>
+      </c>
+      <c r="F1" s="14" t="s">
+        <v>1108</v>
+      </c>
+      <c r="G1" s="14" t="s">
+        <v>1109</v>
+      </c>
+      <c r="H1" s="14" t="s">
+        <v>1110</v>
+      </c>
+      <c r="I1" s="14" t="s">
+        <v>1111</v>
+      </c>
+      <c r="J1" s="14" t="s">
+        <v>1112</v>
+      </c>
+      <c r="K1" s="14" t="s">
+        <v>917</v>
+      </c>
+      <c r="L1" s="14" t="s">
+        <v>1113</v>
+      </c>
+      <c r="M1" s="14" t="s">
+        <v>8</v>
+      </c>
+      <c r="N1" s="14" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="15" t="s">
+        <v>1114</v>
+      </c>
+      <c r="B2" s="15" t="s">
+        <v>1115</v>
+      </c>
+      <c r="C2" s="15" t="s">
+        <v>1116</v>
+      </c>
+      <c r="D2" s="16" t="s">
+        <v>1117</v>
+      </c>
+      <c r="E2" s="15" t="s">
+        <v>1118</v>
+      </c>
+      <c r="F2" s="15" t="s">
+        <v>1119</v>
+      </c>
+      <c r="G2" s="15" t="s">
+        <v>1120</v>
+      </c>
+      <c r="H2" s="15" t="s">
+        <v>1121</v>
+      </c>
+      <c r="I2" s="15" t="s">
+        <v>1122</v>
+      </c>
+      <c r="J2" s="15" t="s">
+        <v>1123</v>
+      </c>
+      <c r="K2" s="18" t="s">
+        <v>925</v>
+      </c>
+      <c r="L2" s="20"/>
+      <c r="M2" s="19" t="s">
+        <v>1124</v>
+      </c>
+      <c r="N2" s="19"/>
+    </row>
+    <row r="3" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="15" t="s">
+        <v>1114</v>
+      </c>
+      <c r="B3" s="15" t="s">
+        <v>1115</v>
+      </c>
+      <c r="C3" s="15" t="s">
+        <v>1116</v>
+      </c>
+      <c r="D3" s="16" t="s">
+        <v>1125</v>
+      </c>
+      <c r="E3" s="15" t="s">
+        <v>1126</v>
+      </c>
+      <c r="F3" s="15" t="s">
+        <v>1127</v>
+      </c>
+      <c r="G3" s="15" t="s">
+        <v>1120</v>
+      </c>
+      <c r="H3" s="15" t="s">
+        <v>1128</v>
+      </c>
+      <c r="I3" s="15" t="s">
+        <v>1129</v>
+      </c>
+      <c r="J3" s="15" t="s">
+        <v>1130</v>
+      </c>
+      <c r="K3" s="18" t="s">
+        <v>925</v>
+      </c>
+      <c r="L3" s="20"/>
+      <c r="M3" s="19" t="s">
+        <v>1124</v>
+      </c>
+      <c r="N3" s="19"/>
+    </row>
+    <row r="4" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="15" t="s">
+        <v>1114</v>
+      </c>
+      <c r="B4" s="15" t="s">
+        <v>1115</v>
+      </c>
+      <c r="C4" s="15" t="s">
+        <v>1131</v>
+      </c>
+      <c r="D4" s="16" t="s">
+        <v>1132</v>
+      </c>
+      <c r="E4" s="15" t="s">
+        <v>1133</v>
+      </c>
+      <c r="F4" s="15" t="s">
+        <v>1134</v>
+      </c>
+      <c r="G4" s="15" t="s">
+        <v>1120</v>
+      </c>
+      <c r="H4" s="15" t="s">
+        <v>1135</v>
+      </c>
+      <c r="I4" s="15" t="s">
+        <v>1136</v>
+      </c>
+      <c r="J4" s="15" t="s">
+        <v>1137</v>
+      </c>
+      <c r="K4" s="18" t="s">
+        <v>925</v>
+      </c>
+      <c r="L4" s="20"/>
+      <c r="M4" s="19" t="s">
+        <v>1124</v>
+      </c>
+      <c r="N4" s="19"/>
+    </row>
+    <row r="5" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="15" t="s">
+        <v>1114</v>
+      </c>
+      <c r="B5" s="15" t="s">
+        <v>1138</v>
+      </c>
+      <c r="C5" s="15" t="s">
+        <v>1139</v>
+      </c>
+      <c r="D5" s="16" t="s">
+        <v>1140</v>
+      </c>
+      <c r="E5" s="15" t="s">
+        <v>1141</v>
+      </c>
+      <c r="F5" s="15" t="s">
+        <v>1142</v>
+      </c>
+      <c r="G5" s="15" t="s">
+        <v>1143</v>
+      </c>
+      <c r="H5" s="15" t="s">
+        <v>1144</v>
+      </c>
+      <c r="I5" s="15"/>
+      <c r="J5" s="15" t="s">
+        <v>1145</v>
+      </c>
+      <c r="K5" s="18" t="s">
+        <v>925</v>
+      </c>
+      <c r="L5" s="20"/>
+      <c r="M5" s="19" t="s">
+        <v>1124</v>
+      </c>
+      <c r="N5" s="19"/>
+    </row>
+    <row r="6" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="15" t="s">
+        <v>1114</v>
+      </c>
+      <c r="B6" s="15" t="s">
+        <v>1138</v>
+      </c>
+      <c r="C6" s="15" t="s">
+        <v>1139</v>
+      </c>
+      <c r="D6" s="16" t="s">
+        <v>1146</v>
+      </c>
+      <c r="E6" s="15" t="s">
+        <v>1147</v>
+      </c>
+      <c r="F6" s="15" t="s">
+        <v>1148</v>
+      </c>
+      <c r="G6" s="15"/>
+      <c r="H6" s="15" t="s">
+        <v>1149</v>
+      </c>
+      <c r="I6" s="15"/>
+      <c r="J6" s="15" t="s">
+        <v>1150</v>
+      </c>
+      <c r="K6" s="18" t="s">
+        <v>925</v>
+      </c>
+      <c r="L6" s="20"/>
+      <c r="M6" s="19" t="s">
+        <v>1124</v>
+      </c>
+      <c r="N6" s="19"/>
+    </row>
+    <row r="7" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="23" t="s">
+        <v>1151</v>
+      </c>
+      <c r="B7" s="23" t="s">
+        <v>1115</v>
+      </c>
+      <c r="C7" s="23" t="s">
+        <v>1116</v>
+      </c>
+      <c r="D7" s="24" t="s">
+        <v>1152</v>
+      </c>
+      <c r="E7" s="23" t="s">
+        <v>1153</v>
+      </c>
+      <c r="F7" s="23" t="s">
+        <v>1154</v>
+      </c>
+      <c r="G7" s="23" t="s">
+        <v>1120</v>
+      </c>
+      <c r="H7" s="23" t="s">
+        <v>939</v>
+      </c>
+      <c r="I7" s="23" t="s">
+        <v>1155</v>
+      </c>
+      <c r="J7" s="23" t="s">
+        <v>1156</v>
+      </c>
+      <c r="K7" s="18" t="s">
+        <v>925</v>
+      </c>
+      <c r="L7" s="20"/>
+      <c r="M7" s="19" t="s">
+        <v>1124</v>
+      </c>
+      <c r="N7" s="19"/>
+    </row>
+    <row r="8" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="23" t="s">
+        <v>1151</v>
+      </c>
+      <c r="B8" s="23" t="s">
+        <v>1115</v>
+      </c>
+      <c r="C8" s="23" t="s">
+        <v>1157</v>
+      </c>
+      <c r="D8" s="24" t="s">
+        <v>1158</v>
+      </c>
+      <c r="E8" s="23" t="s">
+        <v>1159</v>
+      </c>
+      <c r="F8" s="23" t="s">
+        <v>1160</v>
+      </c>
+      <c r="G8" s="23" t="s">
+        <v>1161</v>
+      </c>
+      <c r="H8" s="23" t="s">
+        <v>1162</v>
+      </c>
+      <c r="I8" s="23" t="s">
+        <v>1163</v>
+      </c>
+      <c r="J8" s="23" t="s">
+        <v>1164</v>
+      </c>
+      <c r="K8" s="18" t="s">
+        <v>925</v>
+      </c>
+      <c r="L8" s="20"/>
+      <c r="M8" s="19" t="s">
+        <v>1124</v>
+      </c>
+      <c r="N8" s="19"/>
+    </row>
+    <row r="9" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="23" t="s">
+        <v>1151</v>
+      </c>
+      <c r="B9" s="23" t="s">
+        <v>1115</v>
+      </c>
+      <c r="C9" s="23" t="s">
+        <v>1157</v>
+      </c>
+      <c r="D9" s="24" t="s">
+        <v>1165</v>
+      </c>
+      <c r="E9" s="23" t="s">
+        <v>1166</v>
+      </c>
+      <c r="F9" s="23" t="s">
+        <v>1160</v>
+      </c>
+      <c r="G9" s="23" t="s">
+        <v>1120</v>
+      </c>
+      <c r="H9" s="23" t="s">
+        <v>939</v>
+      </c>
+      <c r="I9" s="23" t="s">
+        <v>1167</v>
+      </c>
+      <c r="J9" s="23" t="s">
+        <v>1168</v>
+      </c>
+      <c r="K9" s="18" t="s">
+        <v>925</v>
+      </c>
+      <c r="L9" s="20"/>
+      <c r="M9" s="19" t="s">
+        <v>1124</v>
+      </c>
+      <c r="N9" s="19"/>
+    </row>
+    <row r="10" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="23" t="s">
+        <v>1151</v>
+      </c>
+      <c r="B10" s="23" t="s">
+        <v>1115</v>
+      </c>
+      <c r="C10" s="23" t="s">
+        <v>1157</v>
+      </c>
+      <c r="D10" s="24" t="s">
+        <v>1169</v>
+      </c>
+      <c r="E10" s="23" t="s">
+        <v>1170</v>
+      </c>
+      <c r="F10" s="23" t="s">
+        <v>1160</v>
+      </c>
+      <c r="G10" s="23" t="s">
+        <v>1161</v>
+      </c>
+      <c r="H10" s="23" t="s">
+        <v>1171</v>
+      </c>
+      <c r="I10" s="23" t="s">
+        <v>1172</v>
+      </c>
+      <c r="J10" s="23" t="s">
+        <v>1173</v>
+      </c>
+      <c r="K10" s="18" t="s">
+        <v>925</v>
+      </c>
+      <c r="L10" s="20"/>
+      <c r="M10" s="19" t="s">
+        <v>1124</v>
+      </c>
+      <c r="N10" s="19"/>
+    </row>
+    <row r="11" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="23" t="s">
+        <v>1151</v>
+      </c>
+      <c r="B11" s="23" t="s">
+        <v>1115</v>
+      </c>
+      <c r="C11" s="23" t="s">
+        <v>1116</v>
+      </c>
+      <c r="D11" s="24" t="s">
+        <v>1174</v>
+      </c>
+      <c r="E11" s="23" t="s">
+        <v>1175</v>
+      </c>
+      <c r="F11" s="23" t="s">
+        <v>1119</v>
+      </c>
+      <c r="G11" s="23" t="s">
+        <v>1176</v>
+      </c>
+      <c r="H11" s="23" t="s">
+        <v>1162</v>
+      </c>
+      <c r="I11" s="23" t="s">
+        <v>1177</v>
+      </c>
+      <c r="J11" s="23" t="s">
+        <v>1178</v>
+      </c>
+      <c r="K11" s="18" t="s">
+        <v>925</v>
+      </c>
+      <c r="L11" s="20"/>
+      <c r="M11" s="19" t="s">
+        <v>1124</v>
+      </c>
+      <c r="N11" s="19"/>
+    </row>
+    <row r="12" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="23" t="s">
+        <v>1151</v>
+      </c>
+      <c r="B12" s="23" t="s">
+        <v>1115</v>
+      </c>
+      <c r="C12" s="23" t="s">
+        <v>1116</v>
+      </c>
+      <c r="D12" s="24" t="s">
+        <v>1179</v>
+      </c>
+      <c r="E12" s="23" t="s">
+        <v>1180</v>
+      </c>
+      <c r="F12" s="23" t="s">
+        <v>1119</v>
+      </c>
+      <c r="G12" s="23" t="s">
+        <v>1120</v>
+      </c>
+      <c r="H12" s="23" t="s">
+        <v>1181</v>
+      </c>
+      <c r="I12" s="23" t="s">
+        <v>1182</v>
+      </c>
+      <c r="J12" s="23" t="s">
+        <v>1183</v>
+      </c>
+      <c r="K12" s="18" t="s">
+        <v>925</v>
+      </c>
+      <c r="L12" s="20"/>
+      <c r="M12" s="19" t="s">
+        <v>1124</v>
+      </c>
+      <c r="N12" s="19"/>
+    </row>
+    <row r="13" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="23" t="s">
+        <v>1151</v>
+      </c>
+      <c r="B13" s="23" t="s">
+        <v>1115</v>
+      </c>
+      <c r="C13" s="23" t="s">
+        <v>1116</v>
+      </c>
+      <c r="D13" s="24" t="s">
+        <v>1184</v>
+      </c>
+      <c r="E13" s="23" t="s">
+        <v>1185</v>
+      </c>
+      <c r="F13" s="23" t="s">
+        <v>1119</v>
+      </c>
+      <c r="G13" s="23" t="s">
+        <v>1120</v>
+      </c>
+      <c r="H13" s="23" t="s">
+        <v>1186</v>
+      </c>
+      <c r="I13" s="23" t="s">
+        <v>1187</v>
+      </c>
+      <c r="J13" s="23" t="s">
+        <v>1188</v>
+      </c>
+      <c r="K13" s="18" t="s">
+        <v>925</v>
+      </c>
+      <c r="L13" s="20"/>
+      <c r="M13" s="19" t="s">
+        <v>1124</v>
+      </c>
+      <c r="N13" s="19"/>
+    </row>
+    <row r="14" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="23" t="s">
+        <v>1151</v>
+      </c>
+      <c r="B14" s="23" t="s">
+        <v>1115</v>
+      </c>
+      <c r="C14" s="23" t="s">
+        <v>1116</v>
+      </c>
+      <c r="D14" s="24" t="s">
+        <v>1189</v>
+      </c>
+      <c r="E14" s="23" t="s">
+        <v>1190</v>
+      </c>
+      <c r="F14" s="23" t="s">
+        <v>1119</v>
+      </c>
+      <c r="G14" s="23" t="s">
+        <v>1191</v>
+      </c>
+      <c r="H14" s="23" t="s">
+        <v>1192</v>
+      </c>
+      <c r="I14" s="23" t="s">
+        <v>1193</v>
+      </c>
+      <c r="J14" s="23" t="s">
+        <v>1194</v>
+      </c>
+      <c r="K14" s="18" t="s">
+        <v>925</v>
+      </c>
+      <c r="L14" s="20"/>
+      <c r="M14" s="19" t="s">
+        <v>1124</v>
+      </c>
+      <c r="N14" s="19"/>
+    </row>
+    <row r="15" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="23" t="s">
+        <v>1151</v>
+      </c>
+      <c r="B15" s="23" t="s">
+        <v>1115</v>
+      </c>
+      <c r="C15" s="23" t="s">
+        <v>1116</v>
+      </c>
+      <c r="D15" s="24" t="s">
+        <v>1195</v>
+      </c>
+      <c r="E15" s="23" t="s">
+        <v>1196</v>
+      </c>
+      <c r="F15" s="23" t="s">
+        <v>1197</v>
+      </c>
+      <c r="G15" s="23" t="s">
+        <v>1120</v>
+      </c>
+      <c r="H15" s="23" t="s">
+        <v>1198</v>
+      </c>
+      <c r="I15" s="23" t="s">
+        <v>1199</v>
+      </c>
+      <c r="J15" s="23" t="s">
+        <v>1200</v>
+      </c>
+      <c r="K15" s="18" t="s">
+        <v>925</v>
+      </c>
+      <c r="L15" s="20"/>
+      <c r="M15" s="19" t="s">
+        <v>1124</v>
+      </c>
+      <c r="N15" s="19"/>
+    </row>
+    <row r="16" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="23" t="s">
+        <v>1151</v>
+      </c>
+      <c r="B16" s="23" t="s">
+        <v>1115</v>
+      </c>
+      <c r="C16" s="23" t="s">
+        <v>1116</v>
+      </c>
+      <c r="D16" s="24" t="s">
+        <v>1201</v>
+      </c>
+      <c r="E16" s="23" t="s">
+        <v>1202</v>
+      </c>
+      <c r="F16" s="23" t="s">
+        <v>1203</v>
+      </c>
+      <c r="G16" s="23" t="s">
+        <v>1204</v>
+      </c>
+      <c r="H16" s="23" t="s">
+        <v>1205</v>
+      </c>
+      <c r="I16" s="23" t="s">
+        <v>1206</v>
+      </c>
+      <c r="J16" s="23" t="s">
+        <v>1207</v>
+      </c>
+      <c r="K16" s="18" t="s">
+        <v>925</v>
+      </c>
+      <c r="L16" s="20"/>
+      <c r="M16" s="19" t="s">
+        <v>1124</v>
+      </c>
+      <c r="N16" s="19"/>
+    </row>
+    <row r="17" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="23" t="s">
+        <v>1151</v>
+      </c>
+      <c r="B17" s="23" t="s">
+        <v>1138</v>
+      </c>
+      <c r="C17" s="23" t="s">
+        <v>1139</v>
+      </c>
+      <c r="D17" s="24" t="s">
+        <v>1208</v>
+      </c>
+      <c r="E17" s="23" t="s">
+        <v>1209</v>
+      </c>
+      <c r="F17" s="23" t="s">
+        <v>1210</v>
+      </c>
+      <c r="G17" s="23" t="s">
+        <v>1211</v>
+      </c>
+      <c r="H17" s="23" t="s">
+        <v>1212</v>
+      </c>
+      <c r="I17" s="23"/>
+      <c r="J17" s="23" t="s">
+        <v>1213</v>
+      </c>
+      <c r="K17" s="18" t="s">
+        <v>925</v>
+      </c>
+      <c r="L17" s="20"/>
+      <c r="M17" s="19" t="s">
+        <v>1124</v>
+      </c>
+      <c r="N17" s="19"/>
+    </row>
+    <row r="18" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="23" t="s">
+        <v>1151</v>
+      </c>
+      <c r="B18" s="23" t="s">
+        <v>1138</v>
+      </c>
+      <c r="C18" s="23" t="s">
+        <v>1139</v>
+      </c>
+      <c r="D18" s="24" t="s">
+        <v>1214</v>
+      </c>
+      <c r="E18" s="23" t="s">
+        <v>1215</v>
+      </c>
+      <c r="F18" s="23" t="s">
+        <v>1216</v>
+      </c>
+      <c r="G18" s="23" t="s">
+        <v>1217</v>
+      </c>
+      <c r="H18" s="23" t="s">
+        <v>1218</v>
+      </c>
+      <c r="I18" s="23"/>
+      <c r="J18" s="23" t="s">
+        <v>1219</v>
+      </c>
+      <c r="K18" s="18" t="s">
+        <v>925</v>
+      </c>
+      <c r="L18" s="20"/>
+      <c r="M18" s="19" t="s">
+        <v>1124</v>
+      </c>
+      <c r="N18" s="19"/>
+    </row>
+    <row r="19" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="23" t="s">
+        <v>1151</v>
+      </c>
+      <c r="B19" s="23" t="s">
+        <v>1138</v>
+      </c>
+      <c r="C19" s="23" t="s">
+        <v>1139</v>
+      </c>
+      <c r="D19" s="24" t="s">
+        <v>1220</v>
+      </c>
+      <c r="E19" s="23" t="s">
+        <v>1221</v>
+      </c>
+      <c r="F19" s="23" t="s">
+        <v>1222</v>
+      </c>
+      <c r="G19" s="23" t="s">
+        <v>1223</v>
+      </c>
+      <c r="H19" s="23" t="s">
+        <v>1224</v>
+      </c>
+      <c r="I19" s="23" t="s">
+        <v>1225</v>
+      </c>
+      <c r="J19" s="23" t="s">
+        <v>1226</v>
+      </c>
+      <c r="K19" s="18" t="s">
+        <v>925</v>
+      </c>
+      <c r="L19" s="20"/>
+      <c r="M19" s="19" t="s">
+        <v>1124</v>
+      </c>
+      <c r="N19" s="19"/>
+    </row>
+    <row r="20" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="23" t="s">
+        <v>1151</v>
+      </c>
+      <c r="B20" s="23" t="s">
+        <v>1138</v>
+      </c>
+      <c r="C20" s="23" t="s">
+        <v>1139</v>
+      </c>
+      <c r="D20" s="24" t="s">
+        <v>1227</v>
+      </c>
+      <c r="E20" s="23" t="s">
+        <v>1228</v>
+      </c>
+      <c r="F20" s="23" t="s">
+        <v>1229</v>
+      </c>
+      <c r="G20" s="23" t="s">
+        <v>1230</v>
+      </c>
+      <c r="H20" s="23" t="s">
+        <v>1224</v>
+      </c>
+      <c r="I20" s="23" t="s">
+        <v>1231</v>
+      </c>
+      <c r="J20" s="23" t="s">
+        <v>1232</v>
+      </c>
+      <c r="K20" s="18" t="s">
+        <v>925</v>
+      </c>
+      <c r="L20" s="20"/>
+      <c r="M20" s="19" t="s">
+        <v>1124</v>
+      </c>
+      <c r="N20" s="19"/>
+    </row>
+    <row r="21" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="23" t="s">
+        <v>1151</v>
+      </c>
+      <c r="B21" s="23" t="s">
+        <v>1138</v>
+      </c>
+      <c r="C21" s="23" t="s">
+        <v>1139</v>
+      </c>
+      <c r="D21" s="24" t="s">
+        <v>1233</v>
+      </c>
+      <c r="E21" s="23" t="s">
+        <v>1234</v>
+      </c>
+      <c r="F21" s="23" t="s">
+        <v>1235</v>
+      </c>
+      <c r="G21" s="23" t="s">
+        <v>1236</v>
+      </c>
+      <c r="H21" s="23"/>
+      <c r="I21" s="23"/>
+      <c r="J21" s="23" t="s">
+        <v>1237</v>
+      </c>
+      <c r="K21" s="18" t="s">
+        <v>925</v>
+      </c>
+      <c r="L21" s="20"/>
+      <c r="M21" s="19" t="s">
+        <v>1124</v>
+      </c>
+      <c r="N21" s="19"/>
+    </row>
+    <row r="22" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="23" t="s">
+        <v>1151</v>
+      </c>
+      <c r="B22" s="23" t="s">
+        <v>1138</v>
+      </c>
+      <c r="C22" s="23" t="s">
+        <v>1139</v>
+      </c>
+      <c r="D22" s="24" t="s">
+        <v>1238</v>
+      </c>
+      <c r="E22" s="23" t="s">
+        <v>1239</v>
+      </c>
+      <c r="F22" s="23"/>
+      <c r="G22" s="23" t="s">
+        <v>1240</v>
+      </c>
+      <c r="H22" s="23" t="s">
+        <v>1241</v>
+      </c>
+      <c r="I22" s="23"/>
+      <c r="J22" s="23" t="s">
+        <v>1242</v>
+      </c>
+      <c r="K22" s="18" t="s">
+        <v>925</v>
+      </c>
+      <c r="L22" s="20"/>
+      <c r="M22" s="19" t="s">
+        <v>1124</v>
+      </c>
+      <c r="N22" s="19"/>
+    </row>
+    <row r="23" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="23" t="s">
+        <v>1151</v>
+      </c>
+      <c r="B23" s="23" t="s">
+        <v>1138</v>
+      </c>
+      <c r="C23" s="23" t="s">
+        <v>1139</v>
+      </c>
+      <c r="D23" s="24" t="s">
+        <v>1243</v>
+      </c>
+      <c r="E23" s="23" t="s">
+        <v>1244</v>
+      </c>
+      <c r="F23" s="23" t="s">
+        <v>1245</v>
+      </c>
+      <c r="G23" s="23" t="s">
+        <v>1246</v>
+      </c>
+      <c r="H23" s="23" t="s">
+        <v>1247</v>
+      </c>
+      <c r="I23" s="23"/>
+      <c r="J23" s="23" t="s">
+        <v>1248</v>
+      </c>
+      <c r="K23" s="18" t="s">
+        <v>925</v>
+      </c>
+      <c r="L23" s="20"/>
+      <c r="M23" s="19" t="s">
+        <v>1124</v>
+      </c>
+      <c r="N23" s="19"/>
+    </row>
+    <row r="24" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="23" t="s">
+        <v>1151</v>
+      </c>
+      <c r="B24" s="23" t="s">
+        <v>1138</v>
+      </c>
+      <c r="C24" s="23" t="s">
+        <v>1139</v>
+      </c>
+      <c r="D24" s="24" t="s">
+        <v>1249</v>
+      </c>
+      <c r="E24" s="23" t="s">
+        <v>1250</v>
+      </c>
+      <c r="F24" s="23" t="s">
+        <v>1251</v>
+      </c>
+      <c r="G24" s="23" t="s">
+        <v>1252</v>
+      </c>
+      <c r="H24" s="23" t="s">
+        <v>1253</v>
+      </c>
+      <c r="I24" s="23"/>
+      <c r="J24" s="23" t="s">
+        <v>1254</v>
+      </c>
+      <c r="K24" s="18" t="s">
+        <v>925</v>
+      </c>
+      <c r="L24" s="20"/>
+      <c r="M24" s="19" t="s">
+        <v>1124</v>
+      </c>
+      <c r="N24" s="19"/>
+    </row>
+    <row r="25" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="23" t="s">
+        <v>1151</v>
+      </c>
+      <c r="B25" s="23" t="s">
+        <v>1138</v>
+      </c>
+      <c r="C25" s="23" t="s">
+        <v>1139</v>
+      </c>
+      <c r="D25" s="24" t="s">
+        <v>1255</v>
+      </c>
+      <c r="E25" s="23" t="s">
+        <v>1256</v>
+      </c>
+      <c r="F25" s="23" t="s">
+        <v>1251</v>
+      </c>
+      <c r="G25" s="23" t="s">
+        <v>1257</v>
+      </c>
+      <c r="H25" s="23" t="s">
+        <v>1258</v>
+      </c>
+      <c r="I25" s="23" t="s">
+        <v>1259</v>
+      </c>
+      <c r="J25" s="23" t="s">
+        <v>1260</v>
+      </c>
+      <c r="K25" s="18" t="s">
+        <v>925</v>
+      </c>
+      <c r="L25" s="20"/>
+      <c r="M25" s="19" t="s">
+        <v>1124</v>
+      </c>
+      <c r="N25" s="19"/>
+    </row>
+    <row r="26" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="23" t="s">
+        <v>1151</v>
+      </c>
+      <c r="B26" s="23" t="s">
+        <v>1138</v>
+      </c>
+      <c r="C26" s="23" t="s">
+        <v>1139</v>
+      </c>
+      <c r="D26" s="24" t="s">
+        <v>1261</v>
+      </c>
+      <c r="E26" s="23" t="s">
+        <v>1262</v>
+      </c>
+      <c r="F26" s="23" t="s">
+        <v>1263</v>
+      </c>
+      <c r="G26" s="23" t="s">
+        <v>1264</v>
+      </c>
+      <c r="H26" s="23"/>
+      <c r="I26" s="23"/>
+      <c r="J26" s="23" t="s">
+        <v>1265</v>
+      </c>
+      <c r="K26" s="18" t="s">
+        <v>925</v>
+      </c>
+      <c r="L26" s="20"/>
+      <c r="M26" s="19" t="s">
+        <v>1124</v>
+      </c>
+      <c r="N26" s="19"/>
+    </row>
+    <row r="27" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="23" t="s">
+        <v>1151</v>
+      </c>
+      <c r="B27" s="23" t="s">
+        <v>1138</v>
+      </c>
+      <c r="C27" s="23" t="s">
+        <v>1139</v>
+      </c>
+      <c r="D27" s="24" t="s">
+        <v>1266</v>
+      </c>
+      <c r="E27" s="23" t="s">
+        <v>1267</v>
+      </c>
+      <c r="F27" s="23" t="s">
+        <v>1268</v>
+      </c>
+      <c r="G27" s="23"/>
+      <c r="H27" s="23"/>
+      <c r="I27" s="23"/>
+      <c r="J27" s="23" t="s">
+        <v>1269</v>
+      </c>
+      <c r="K27" s="18" t="s">
+        <v>925</v>
+      </c>
+      <c r="L27" s="20"/>
+      <c r="M27" s="19" t="s">
+        <v>1124</v>
+      </c>
+      <c r="N27" s="19"/>
+    </row>
+    <row r="28" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="23" t="s">
+        <v>1151</v>
+      </c>
+      <c r="B28" s="23" t="s">
+        <v>1138</v>
+      </c>
+      <c r="C28" s="23" t="s">
+        <v>1139</v>
+      </c>
+      <c r="D28" s="24" t="s">
+        <v>1270</v>
+      </c>
+      <c r="E28" s="23" t="s">
+        <v>1271</v>
+      </c>
+      <c r="F28" s="23" t="s">
+        <v>1272</v>
+      </c>
+      <c r="G28" s="23"/>
+      <c r="H28" s="23" t="s">
+        <v>939</v>
+      </c>
+      <c r="I28" s="23" t="s">
+        <v>1273</v>
+      </c>
+      <c r="J28" s="23" t="s">
+        <v>1274</v>
+      </c>
+      <c r="K28" s="18" t="s">
+        <v>925</v>
+      </c>
+      <c r="L28" s="20"/>
+      <c r="M28" s="19" t="s">
+        <v>1124</v>
+      </c>
+      <c r="N28" s="19"/>
+    </row>
+    <row r="29" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="23" t="s">
+        <v>1151</v>
+      </c>
+      <c r="B29" s="23" t="s">
+        <v>1138</v>
+      </c>
+      <c r="C29" s="23" t="s">
+        <v>1139</v>
+      </c>
+      <c r="D29" s="24" t="s">
+        <v>1275</v>
+      </c>
+      <c r="E29" s="23" t="s">
+        <v>1276</v>
+      </c>
+      <c r="F29" s="23"/>
+      <c r="G29" s="23"/>
+      <c r="H29" s="23" t="s">
+        <v>939</v>
+      </c>
+      <c r="I29" s="23" t="s">
+        <v>1277</v>
+      </c>
+      <c r="J29" s="23" t="s">
+        <v>1278</v>
+      </c>
+      <c r="K29" s="18" t="s">
+        <v>925</v>
+      </c>
+      <c r="L29" s="20"/>
+      <c r="M29" s="19" t="s">
+        <v>1124</v>
+      </c>
+      <c r="N29" s="19"/>
+    </row>
+    <row r="30" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="23" t="s">
+        <v>1151</v>
+      </c>
+      <c r="B30" s="23" t="s">
+        <v>1138</v>
+      </c>
+      <c r="C30" s="23" t="s">
+        <v>1139</v>
+      </c>
+      <c r="D30" s="24" t="s">
+        <v>1279</v>
+      </c>
+      <c r="E30" s="23" t="s">
+        <v>1280</v>
+      </c>
+      <c r="F30" s="23" t="s">
+        <v>1281</v>
+      </c>
+      <c r="G30" s="23" t="s">
+        <v>1282</v>
+      </c>
+      <c r="H30" s="23" t="s">
+        <v>1283</v>
+      </c>
+      <c r="I30" s="23" t="s">
+        <v>1284</v>
+      </c>
+      <c r="J30" s="23" t="s">
+        <v>1285</v>
+      </c>
+      <c r="K30" s="18" t="s">
+        <v>925</v>
+      </c>
+      <c r="L30" s="20"/>
+      <c r="M30" s="19" t="s">
+        <v>1124</v>
+      </c>
+      <c r="N30" s="19"/>
+    </row>
+    <row r="31" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="17" t="s">
+        <v>1286</v>
+      </c>
+      <c r="B31" s="17" t="s">
+        <v>1287</v>
+      </c>
+      <c r="C31" s="17" t="s">
+        <v>1116</v>
+      </c>
+      <c r="D31" s="25" t="s">
+        <v>1288</v>
+      </c>
+      <c r="E31" s="17" t="s">
+        <v>1289</v>
+      </c>
+      <c r="F31" s="17" t="s">
+        <v>1119</v>
+      </c>
+      <c r="G31" s="17" t="s">
+        <v>1290</v>
+      </c>
+      <c r="H31" s="17" t="s">
+        <v>1291</v>
+      </c>
+      <c r="I31" s="17" t="s">
+        <v>1292</v>
+      </c>
+      <c r="J31" s="17" t="s">
+        <v>1293</v>
+      </c>
+      <c r="K31" s="18" t="s">
+        <v>925</v>
+      </c>
+      <c r="L31" s="20"/>
+      <c r="M31" s="19" t="s">
+        <v>1124</v>
+      </c>
+      <c r="N31" s="19"/>
+    </row>
+    <row r="32" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="17" t="s">
+        <v>1286</v>
+      </c>
+      <c r="B32" s="17" t="s">
+        <v>1115</v>
+      </c>
+      <c r="C32" s="17" t="s">
+        <v>1116</v>
+      </c>
+      <c r="D32" s="25" t="s">
+        <v>1294</v>
+      </c>
+      <c r="E32" s="17" t="s">
+        <v>1295</v>
+      </c>
+      <c r="F32" s="17" t="s">
+        <v>1296</v>
+      </c>
+      <c r="G32" s="17" t="s">
+        <v>1297</v>
+      </c>
+      <c r="H32" s="17" t="s">
+        <v>1298</v>
+      </c>
+      <c r="I32" s="17" t="s">
+        <v>1299</v>
+      </c>
+      <c r="J32" s="17" t="s">
+        <v>1300</v>
+      </c>
+      <c r="K32" s="18" t="s">
+        <v>925</v>
+      </c>
+      <c r="L32" s="20"/>
+      <c r="M32" s="19" t="s">
+        <v>1124</v>
+      </c>
+      <c r="N32" s="19"/>
+    </row>
+    <row r="33" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="17" t="s">
+        <v>1286</v>
+      </c>
+      <c r="B33" s="17" t="s">
+        <v>1115</v>
+      </c>
+      <c r="C33" s="17" t="s">
+        <v>1131</v>
+      </c>
+      <c r="D33" s="25" t="s">
+        <v>1301</v>
+      </c>
+      <c r="E33" s="17" t="s">
+        <v>1302</v>
+      </c>
+      <c r="F33" s="17" t="s">
+        <v>1303</v>
+      </c>
+      <c r="G33" s="17" t="s">
+        <v>1304</v>
+      </c>
+      <c r="H33" s="17" t="s">
+        <v>1305</v>
+      </c>
+      <c r="I33" s="17" t="s">
+        <v>1306</v>
+      </c>
+      <c r="J33" s="17" t="s">
+        <v>1307</v>
+      </c>
+      <c r="K33" s="18" t="s">
+        <v>925</v>
+      </c>
+      <c r="L33" s="20"/>
+      <c r="M33" s="19" t="s">
+        <v>1124</v>
+      </c>
+      <c r="N33" s="19"/>
+    </row>
+    <row r="34" customFormat="false" ht="79.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="17" t="s">
+        <v>1286</v>
+      </c>
+      <c r="B34" s="17" t="s">
+        <v>1287</v>
+      </c>
+      <c r="C34" s="17" t="s">
+        <v>1131</v>
+      </c>
+      <c r="D34" s="25" t="s">
+        <v>1308</v>
+      </c>
+      <c r="E34" s="17" t="s">
+        <v>1309</v>
+      </c>
+      <c r="F34" s="17" t="s">
+        <v>1310</v>
+      </c>
+      <c r="G34" s="17" t="s">
+        <v>1120</v>
+      </c>
+      <c r="H34" s="17" t="s">
+        <v>1311</v>
+      </c>
+      <c r="I34" s="17" t="s">
+        <v>1312</v>
+      </c>
+      <c r="J34" s="17" t="s">
+        <v>1313</v>
+      </c>
+      <c r="K34" s="18" t="s">
+        <v>925</v>
+      </c>
+      <c r="L34" s="20"/>
+      <c r="M34" s="19" t="s">
+        <v>1124</v>
+      </c>
+      <c r="N34" s="19"/>
+    </row>
+    <row r="35" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="17" t="s">
+        <v>1286</v>
+      </c>
+      <c r="B35" s="17" t="s">
+        <v>1287</v>
+      </c>
+      <c r="C35" s="17" t="s">
+        <v>1131</v>
+      </c>
+      <c r="D35" s="25" t="s">
+        <v>1314</v>
+      </c>
+      <c r="E35" s="17" t="s">
+        <v>1315</v>
+      </c>
+      <c r="F35" s="17" t="s">
+        <v>1148</v>
+      </c>
+      <c r="G35" s="17" t="s">
+        <v>1316</v>
+      </c>
+      <c r="H35" s="17" t="s">
+        <v>1291</v>
+      </c>
+      <c r="I35" s="17" t="s">
+        <v>1317</v>
+      </c>
+      <c r="J35" s="17" t="s">
+        <v>1318</v>
+      </c>
+      <c r="K35" s="18" t="s">
+        <v>925</v>
+      </c>
+      <c r="L35" s="20"/>
+      <c r="M35" s="19" t="s">
+        <v>1124</v>
+      </c>
+      <c r="N35" s="19"/>
+    </row>
+    <row r="36" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="17" t="s">
+        <v>1286</v>
+      </c>
+      <c r="B36" s="17" t="s">
+        <v>1115</v>
+      </c>
+      <c r="C36" s="17" t="s">
+        <v>1319</v>
+      </c>
+      <c r="D36" s="25" t="s">
+        <v>1320</v>
+      </c>
+      <c r="E36" s="17" t="s">
+        <v>1321</v>
+      </c>
+      <c r="F36" s="17" t="s">
+        <v>1322</v>
+      </c>
+      <c r="G36" s="17" t="s">
+        <v>1323</v>
+      </c>
+      <c r="H36" s="17" t="s">
+        <v>939</v>
+      </c>
+      <c r="I36" s="17" t="s">
+        <v>1324</v>
+      </c>
+      <c r="J36" s="17" t="s">
+        <v>1325</v>
+      </c>
+      <c r="K36" s="18" t="s">
+        <v>925</v>
+      </c>
+      <c r="L36" s="20"/>
+      <c r="M36" s="19" t="s">
+        <v>1124</v>
+      </c>
+      <c r="N36" s="19"/>
+    </row>
+    <row r="37" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="17" t="s">
+        <v>1286</v>
+      </c>
+      <c r="B37" s="17" t="s">
+        <v>1115</v>
+      </c>
+      <c r="C37" s="17" t="s">
+        <v>1319</v>
+      </c>
+      <c r="D37" s="25" t="s">
+        <v>1326</v>
+      </c>
+      <c r="E37" s="17" t="s">
+        <v>1327</v>
+      </c>
+      <c r="F37" s="17" t="s">
+        <v>1119</v>
+      </c>
+      <c r="G37" s="17" t="s">
+        <v>1120</v>
+      </c>
+      <c r="H37" s="17" t="s">
+        <v>1328</v>
+      </c>
+      <c r="I37" s="17" t="s">
+        <v>1329</v>
+      </c>
+      <c r="J37" s="17" t="s">
+        <v>1330</v>
+      </c>
+      <c r="K37" s="18" t="s">
+        <v>925</v>
+      </c>
+      <c r="L37" s="20"/>
+      <c r="M37" s="19" t="s">
+        <v>1124</v>
+      </c>
+      <c r="N37" s="19"/>
+    </row>
+    <row r="38" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="17" t="s">
+        <v>1286</v>
+      </c>
+      <c r="B38" s="17" t="s">
+        <v>1115</v>
+      </c>
+      <c r="C38" s="17" t="s">
+        <v>1157</v>
+      </c>
+      <c r="D38" s="25" t="s">
+        <v>1331</v>
+      </c>
+      <c r="E38" s="17" t="s">
+        <v>1332</v>
+      </c>
+      <c r="F38" s="17" t="s">
+        <v>1333</v>
+      </c>
+      <c r="G38" s="17" t="s">
+        <v>1334</v>
+      </c>
+      <c r="H38" s="17" t="s">
+        <v>1335</v>
+      </c>
+      <c r="I38" s="17" t="s">
+        <v>1336</v>
+      </c>
+      <c r="J38" s="17" t="s">
+        <v>1337</v>
+      </c>
+      <c r="K38" s="18" t="s">
+        <v>925</v>
+      </c>
+      <c r="L38" s="20"/>
+      <c r="M38" s="19" t="s">
+        <v>1124</v>
+      </c>
+      <c r="N38" s="19"/>
+    </row>
+    <row r="39" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="17" t="s">
+        <v>1286</v>
+      </c>
+      <c r="B39" s="17" t="s">
+        <v>1115</v>
+      </c>
+      <c r="C39" s="17" t="s">
+        <v>1157</v>
+      </c>
+      <c r="D39" s="25" t="s">
+        <v>1338</v>
+      </c>
+      <c r="E39" s="17" t="s">
+        <v>1339</v>
+      </c>
+      <c r="F39" s="17" t="s">
+        <v>1160</v>
+      </c>
+      <c r="G39" s="17" t="s">
+        <v>1161</v>
+      </c>
+      <c r="H39" s="17" t="s">
+        <v>1340</v>
+      </c>
+      <c r="I39" s="17" t="s">
+        <v>1341</v>
+      </c>
+      <c r="J39" s="17" t="s">
+        <v>1342</v>
+      </c>
+      <c r="K39" s="18" t="s">
+        <v>925</v>
+      </c>
+      <c r="L39" s="20"/>
+      <c r="M39" s="19" t="s">
+        <v>1124</v>
+      </c>
+      <c r="N39" s="19"/>
+    </row>
+    <row r="40" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="17" t="s">
+        <v>1286</v>
+      </c>
+      <c r="B40" s="17" t="s">
+        <v>1115</v>
+      </c>
+      <c r="C40" s="17" t="s">
+        <v>1116</v>
+      </c>
+      <c r="D40" s="25" t="s">
+        <v>1343</v>
+      </c>
+      <c r="E40" s="17" t="s">
+        <v>1344</v>
+      </c>
+      <c r="F40" s="17" t="s">
+        <v>1345</v>
+      </c>
+      <c r="G40" s="17" t="s">
+        <v>1346</v>
+      </c>
+      <c r="H40" s="17" t="s">
+        <v>1328</v>
+      </c>
+      <c r="I40" s="17" t="s">
+        <v>1347</v>
+      </c>
+      <c r="J40" s="17" t="s">
+        <v>1348</v>
+      </c>
+      <c r="K40" s="18" t="s">
+        <v>925</v>
+      </c>
+      <c r="L40" s="20"/>
+      <c r="M40" s="19" t="s">
+        <v>1124</v>
+      </c>
+      <c r="N40" s="19"/>
+    </row>
+    <row r="41" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="17" t="s">
+        <v>1286</v>
+      </c>
+      <c r="B41" s="17" t="s">
+        <v>1138</v>
+      </c>
+      <c r="C41" s="17" t="s">
+        <v>1139</v>
+      </c>
+      <c r="D41" s="25" t="s">
+        <v>1349</v>
+      </c>
+      <c r="E41" s="17" t="s">
+        <v>1350</v>
+      </c>
+      <c r="F41" s="17"/>
+      <c r="G41" s="17" t="s">
+        <v>1351</v>
+      </c>
+      <c r="H41" s="17" t="s">
+        <v>939</v>
+      </c>
+      <c r="I41" s="17" t="s">
+        <v>1352</v>
+      </c>
+      <c r="J41" s="17" t="s">
+        <v>1353</v>
+      </c>
+      <c r="K41" s="18" t="s">
+        <v>925</v>
+      </c>
+      <c r="L41" s="20"/>
+      <c r="M41" s="19" t="s">
+        <v>1124</v>
+      </c>
+      <c r="N41" s="19"/>
+    </row>
+    <row r="42" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="17" t="s">
+        <v>1286</v>
+      </c>
+      <c r="B42" s="17" t="s">
+        <v>1138</v>
+      </c>
+      <c r="C42" s="17" t="s">
+        <v>1139</v>
+      </c>
+      <c r="D42" s="25" t="s">
+        <v>1354</v>
+      </c>
+      <c r="E42" s="17" t="s">
+        <v>1355</v>
+      </c>
+      <c r="F42" s="17" t="s">
+        <v>1356</v>
+      </c>
+      <c r="G42" s="17"/>
+      <c r="H42" s="17" t="s">
+        <v>1357</v>
+      </c>
+      <c r="I42" s="17" t="s">
+        <v>1358</v>
+      </c>
+      <c r="J42" s="17" t="s">
+        <v>1359</v>
+      </c>
+      <c r="K42" s="18" t="s">
+        <v>925</v>
+      </c>
+      <c r="L42" s="20"/>
+      <c r="M42" s="19" t="s">
+        <v>1124</v>
+      </c>
+      <c r="N42" s="19"/>
+    </row>
+    <row r="43" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="17" t="s">
+        <v>1286</v>
+      </c>
+      <c r="B43" s="17" t="s">
+        <v>1138</v>
+      </c>
+      <c r="C43" s="17" t="s">
+        <v>1139</v>
+      </c>
+      <c r="D43" s="25" t="s">
+        <v>1360</v>
+      </c>
+      <c r="E43" s="17" t="s">
+        <v>1361</v>
+      </c>
+      <c r="F43" s="17"/>
+      <c r="G43" s="17" t="s">
+        <v>1362</v>
+      </c>
+      <c r="H43" s="17" t="s">
+        <v>1311</v>
+      </c>
+      <c r="I43" s="17" t="s">
+        <v>1363</v>
+      </c>
+      <c r="J43" s="17" t="s">
+        <v>1364</v>
+      </c>
+      <c r="K43" s="18" t="s">
+        <v>925</v>
+      </c>
+      <c r="L43" s="20"/>
+      <c r="M43" s="19" t="s">
+        <v>1124</v>
+      </c>
+      <c r="N43" s="19"/>
+    </row>
+    <row r="44" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="17" t="s">
+        <v>1286</v>
+      </c>
+      <c r="B44" s="17" t="s">
+        <v>1138</v>
+      </c>
+      <c r="C44" s="17" t="s">
+        <v>1139</v>
+      </c>
+      <c r="D44" s="25" t="s">
+        <v>1365</v>
+      </c>
+      <c r="E44" s="17" t="s">
+        <v>1366</v>
+      </c>
+      <c r="F44" s="17" t="s">
+        <v>1367</v>
+      </c>
+      <c r="G44" s="17" t="s">
+        <v>1368</v>
+      </c>
+      <c r="H44" s="17" t="s">
+        <v>1369</v>
+      </c>
+      <c r="I44" s="17" t="s">
+        <v>1370</v>
+      </c>
+      <c r="J44" s="17" t="s">
+        <v>1371</v>
+      </c>
+      <c r="K44" s="18" t="s">
+        <v>925</v>
+      </c>
+      <c r="L44" s="20"/>
+      <c r="M44" s="19" t="s">
+        <v>1124</v>
+      </c>
+      <c r="N44" s="19"/>
+    </row>
+    <row r="45" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="17" t="s">
+        <v>1286</v>
+      </c>
+      <c r="B45" s="17" t="s">
+        <v>1138</v>
+      </c>
+      <c r="C45" s="17" t="s">
+        <v>1139</v>
+      </c>
+      <c r="D45" s="25" t="s">
+        <v>1372</v>
+      </c>
+      <c r="E45" s="17" t="s">
+        <v>1373</v>
+      </c>
+      <c r="F45" s="17"/>
+      <c r="G45" s="17" t="s">
+        <v>1374</v>
+      </c>
+      <c r="H45" s="17" t="s">
+        <v>1375</v>
+      </c>
+      <c r="I45" s="17" t="s">
+        <v>1376</v>
+      </c>
+      <c r="J45" s="17" t="s">
+        <v>1377</v>
+      </c>
+      <c r="K45" s="18" t="s">
+        <v>925</v>
+      </c>
+      <c r="L45" s="20"/>
+      <c r="M45" s="19" t="s">
+        <v>1124</v>
+      </c>
+      <c r="N45" s="19"/>
+    </row>
+    <row r="46" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="17" t="s">
+        <v>1286</v>
+      </c>
+      <c r="B46" s="17" t="s">
+        <v>1138</v>
+      </c>
+      <c r="C46" s="17" t="s">
+        <v>1139</v>
+      </c>
+      <c r="D46" s="25" t="s">
+        <v>1378</v>
+      </c>
+      <c r="E46" s="17" t="s">
+        <v>1379</v>
+      </c>
+      <c r="F46" s="17" t="s">
+        <v>1380</v>
+      </c>
+      <c r="G46" s="17" t="s">
+        <v>1381</v>
+      </c>
+      <c r="H46" s="17" t="s">
+        <v>1382</v>
+      </c>
+      <c r="I46" s="17" t="s">
+        <v>1383</v>
+      </c>
+      <c r="J46" s="17" t="s">
+        <v>1384</v>
+      </c>
+      <c r="K46" s="18" t="s">
+        <v>925</v>
+      </c>
+      <c r="L46" s="20"/>
+      <c r="M46" s="19" t="s">
+        <v>1124</v>
+      </c>
+      <c r="N46" s="19"/>
+    </row>
+    <row r="47" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="17" t="s">
+        <v>1286</v>
+      </c>
+      <c r="B47" s="17" t="s">
+        <v>1138</v>
+      </c>
+      <c r="C47" s="17" t="s">
+        <v>1139</v>
+      </c>
+      <c r="D47" s="25" t="s">
+        <v>1385</v>
+      </c>
+      <c r="E47" s="17" t="s">
+        <v>1386</v>
+      </c>
+      <c r="F47" s="17" t="s">
+        <v>1127</v>
+      </c>
+      <c r="G47" s="17" t="s">
+        <v>1387</v>
+      </c>
+      <c r="H47" s="17" t="s">
+        <v>1382</v>
+      </c>
+      <c r="I47" s="17" t="s">
+        <v>1388</v>
+      </c>
+      <c r="J47" s="17" t="s">
+        <v>1389</v>
+      </c>
+      <c r="K47" s="18" t="s">
+        <v>925</v>
+      </c>
+      <c r="L47" s="20"/>
+      <c r="M47" s="19" t="s">
+        <v>1124</v>
+      </c>
+      <c r="N47" s="19"/>
+    </row>
+    <row r="48" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="17" t="s">
+        <v>1286</v>
+      </c>
+      <c r="B48" s="17" t="s">
+        <v>1138</v>
+      </c>
+      <c r="C48" s="17" t="s">
+        <v>1139</v>
+      </c>
+      <c r="D48" s="25" t="s">
+        <v>1390</v>
+      </c>
+      <c r="E48" s="17" t="s">
+        <v>1391</v>
+      </c>
+      <c r="F48" s="17" t="s">
+        <v>1392</v>
+      </c>
+      <c r="G48" s="17" t="s">
+        <v>1393</v>
+      </c>
+      <c r="H48" s="17" t="s">
+        <v>1394</v>
+      </c>
+      <c r="I48" s="17" t="s">
+        <v>1376</v>
+      </c>
+      <c r="J48" s="17" t="s">
+        <v>1395</v>
+      </c>
+      <c r="K48" s="18" t="s">
+        <v>925</v>
+      </c>
+      <c r="L48" s="20"/>
+      <c r="M48" s="19" t="s">
+        <v>1124</v>
+      </c>
+      <c r="N48" s="19"/>
+    </row>
+    <row r="49" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="17" t="s">
+        <v>1286</v>
+      </c>
+      <c r="B49" s="17" t="s">
+        <v>1138</v>
+      </c>
+      <c r="C49" s="17" t="s">
+        <v>1139</v>
+      </c>
+      <c r="D49" s="25" t="s">
+        <v>1396</v>
+      </c>
+      <c r="E49" s="17" t="s">
+        <v>1397</v>
+      </c>
+      <c r="F49" s="17" t="s">
+        <v>1398</v>
+      </c>
+      <c r="G49" s="17" t="s">
+        <v>1399</v>
+      </c>
+      <c r="H49" s="17" t="s">
+        <v>1400</v>
+      </c>
+      <c r="I49" s="17" t="s">
+        <v>1401</v>
+      </c>
+      <c r="J49" s="17" t="s">
+        <v>1402</v>
+      </c>
+      <c r="K49" s="18" t="s">
+        <v>925</v>
+      </c>
+      <c r="L49" s="20"/>
+      <c r="M49" s="19" t="s">
+        <v>1124</v>
+      </c>
+      <c r="N49" s="19"/>
+    </row>
+    <row r="50" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A50" s="17" t="s">
+        <v>1286</v>
+      </c>
+      <c r="B50" s="17" t="s">
+        <v>1138</v>
+      </c>
+      <c r="C50" s="17" t="s">
+        <v>1139</v>
+      </c>
+      <c r="D50" s="25" t="s">
+        <v>1403</v>
+      </c>
+      <c r="E50" s="17" t="s">
+        <v>1404</v>
+      </c>
+      <c r="F50" s="17" t="s">
+        <v>1405</v>
+      </c>
+      <c r="G50" s="17" t="s">
+        <v>1406</v>
+      </c>
+      <c r="H50" s="17" t="s">
+        <v>1407</v>
+      </c>
+      <c r="I50" s="17" t="s">
+        <v>1408</v>
+      </c>
+      <c r="J50" s="17" t="s">
+        <v>1409</v>
+      </c>
+      <c r="K50" s="18" t="s">
+        <v>925</v>
+      </c>
+      <c r="L50" s="20"/>
+      <c r="M50" s="19" t="s">
+        <v>1124</v>
+      </c>
+      <c r="N50" s="19"/>
+    </row>
+    <row r="51" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A51" s="17" t="s">
+        <v>1286</v>
+      </c>
+      <c r="B51" s="17" t="s">
+        <v>1138</v>
+      </c>
+      <c r="C51" s="17" t="s">
+        <v>1139</v>
+      </c>
+      <c r="D51" s="25" t="s">
+        <v>1410</v>
+      </c>
+      <c r="E51" s="17" t="s">
+        <v>1411</v>
+      </c>
+      <c r="F51" s="17" t="s">
+        <v>1412</v>
+      </c>
+      <c r="G51" s="17" t="s">
+        <v>1413</v>
+      </c>
+      <c r="H51" s="17"/>
+      <c r="I51" s="17" t="s">
+        <v>1414</v>
+      </c>
+      <c r="J51" s="17" t="s">
+        <v>1415</v>
+      </c>
+      <c r="K51" s="18" t="s">
+        <v>925</v>
+      </c>
+      <c r="L51" s="20"/>
+      <c r="M51" s="19" t="s">
+        <v>1124</v>
+      </c>
+      <c r="N51" s="19"/>
+    </row>
+    <row r="52" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A52" s="17" t="s">
+        <v>1286</v>
+      </c>
+      <c r="B52" s="17" t="s">
+        <v>1138</v>
+      </c>
+      <c r="C52" s="17" t="s">
+        <v>1139</v>
+      </c>
+      <c r="D52" s="25" t="s">
+        <v>1416</v>
+      </c>
+      <c r="E52" s="17" t="s">
+        <v>1417</v>
+      </c>
+      <c r="F52" s="17"/>
+      <c r="G52" s="17" t="s">
+        <v>1418</v>
+      </c>
+      <c r="H52" s="17" t="s">
+        <v>1419</v>
+      </c>
+      <c r="I52" s="17" t="s">
+        <v>1420</v>
+      </c>
+      <c r="J52" s="17" t="s">
+        <v>1421</v>
+      </c>
+      <c r="K52" s="18" t="s">
+        <v>925</v>
+      </c>
+      <c r="L52" s="20"/>
+      <c r="M52" s="19" t="s">
+        <v>1124</v>
+      </c>
+      <c r="N52" s="19"/>
+    </row>
+    <row r="53" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A53" s="17" t="s">
+        <v>1286</v>
+      </c>
+      <c r="B53" s="17" t="s">
+        <v>1138</v>
+      </c>
+      <c r="C53" s="17" t="s">
+        <v>1139</v>
+      </c>
+      <c r="D53" s="25" t="s">
+        <v>1422</v>
+      </c>
+      <c r="E53" s="17" t="s">
+        <v>1423</v>
+      </c>
+      <c r="F53" s="17"/>
+      <c r="G53" s="17" t="s">
+        <v>1424</v>
+      </c>
+      <c r="H53" s="17" t="s">
+        <v>1425</v>
+      </c>
+      <c r="I53" s="17"/>
+      <c r="J53" s="17" t="s">
+        <v>1426</v>
+      </c>
+      <c r="K53" s="18" t="s">
+        <v>925</v>
+      </c>
+      <c r="L53" s="20"/>
+      <c r="M53" s="19" t="s">
+        <v>1124</v>
+      </c>
+      <c r="N53" s="19"/>
+    </row>
+    <row r="55" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A55" s="2" t="s">
+        <v>1427</v>
+      </c>
+      <c r="B55" s="2"/>
+      <c r="C55" s="2"/>
+      <c r="D55" s="2"/>
+      <c r="E55" s="2"/>
+      <c r="F55" s="2"/>
+      <c r="G55" s="2"/>
+      <c r="H55" s="2"/>
+      <c r="I55" s="2"/>
+      <c r="J55" s="2"/>
+    </row>
+    <row r="56" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A56" s="2" t="s">
+        <v>1428</v>
+      </c>
+      <c r="B56" s="2"/>
+      <c r="C56" s="2"/>
+      <c r="D56" s="2"/>
+      <c r="E56" s="2"/>
+      <c r="F56" s="2"/>
+      <c r="G56" s="2"/>
+      <c r="H56" s="2"/>
+      <c r="I56" s="2"/>
+      <c r="J56" s="2"/>
+    </row>
+    <row r="57" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A57" s="2" t="s">
+        <v>1429</v>
+      </c>
+      <c r="B57" s="2"/>
+      <c r="C57" s="2"/>
+      <c r="D57" s="2"/>
+      <c r="E57" s="2"/>
+      <c r="F57" s="2"/>
+      <c r="G57" s="2"/>
+      <c r="H57" s="2"/>
+      <c r="I57" s="2"/>
+      <c r="J57" s="2"/>
+    </row>
+    <row r="58" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A58" s="2" t="s">
+        <v>1430</v>
+      </c>
+      <c r="B58" s="2"/>
+      <c r="C58" s="2"/>
+      <c r="D58" s="2"/>
+      <c r="E58" s="2"/>
+      <c r="F58" s="2"/>
+      <c r="G58" s="2"/>
+      <c r="H58" s="2"/>
+      <c r="I58" s="2"/>
+      <c r="J58" s="2"/>
+    </row>
+    <row r="59" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A59" s="2" t="s">
+        <v>1431</v>
+      </c>
+      <c r="B59" s="2"/>
+      <c r="C59" s="2"/>
+      <c r="D59" s="2"/>
+      <c r="E59" s="2"/>
+      <c r="F59" s="2"/>
+      <c r="G59" s="2"/>
+      <c r="H59" s="2"/>
+      <c r="I59" s="2"/>
+      <c r="J59" s="2"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:N53"/>
+  <mergeCells count="5">
+    <mergeCell ref="A55:J55"/>
+    <mergeCell ref="A56:J56"/>
+    <mergeCell ref="A57:J57"/>
+    <mergeCell ref="A58:J58"/>
+    <mergeCell ref="A59:J59"/>
+  </mergeCells>
+  <dataValidations count="1">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="M2:M132" type="list">
+      <formula1>"À étudier,Répondu,Pas pertinent,Gagné,Perdu"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+  </dataValidations>
+  <hyperlinks>
+    <hyperlink ref="K2" r:id="rId1" display="Ouvrir"/>
+    <hyperlink ref="K3" r:id="rId2" display="Ouvrir"/>
+    <hyperlink ref="K4" r:id="rId3" display="Ouvrir"/>
+    <hyperlink ref="K5" r:id="rId4" display="Ouvrir"/>
+    <hyperlink ref="K6" r:id="rId5" display="Ouvrir"/>
+    <hyperlink ref="K7" r:id="rId6" display="Ouvrir"/>
+    <hyperlink ref="K8" r:id="rId7" display="Ouvrir"/>
+    <hyperlink ref="K9" r:id="rId8" display="Ouvrir"/>
+    <hyperlink ref="K10" r:id="rId9" display="Ouvrir"/>
+    <hyperlink ref="K11" r:id="rId10" display="Ouvrir"/>
+    <hyperlink ref="K12" r:id="rId11" display="Ouvrir"/>
+    <hyperlink ref="K13" r:id="rId12" display="Ouvrir"/>
+    <hyperlink ref="K14" r:id="rId13" display="Ouvrir"/>
+    <hyperlink ref="K15" r:id="rId14" display="Ouvrir"/>
+    <hyperlink ref="K16" r:id="rId15" display="Ouvrir"/>
+    <hyperlink ref="K17" r:id="rId16" display="Ouvrir"/>
+    <hyperlink ref="K18" r:id="rId17" display="Ouvrir"/>
+    <hyperlink ref="K19" r:id="rId18" display="Ouvrir"/>
+    <hyperlink ref="K20" r:id="rId19" display="Ouvrir"/>
+    <hyperlink ref="K21" r:id="rId20" display="Ouvrir"/>
+    <hyperlink ref="K22" r:id="rId21" display="Ouvrir"/>
+    <hyperlink ref="K23" r:id="rId22" display="Ouvrir"/>
+    <hyperlink ref="K24" r:id="rId23" display="Ouvrir"/>
+    <hyperlink ref="K25" r:id="rId24" display="Ouvrir"/>
+    <hyperlink ref="K26" r:id="rId25" display="Ouvrir"/>
+    <hyperlink ref="K27" r:id="rId26" display="Ouvrir"/>
+    <hyperlink ref="K28" r:id="rId27" display="Ouvrir"/>
+    <hyperlink ref="K29" r:id="rId28" display="Ouvrir"/>
+    <hyperlink ref="K30" r:id="rId29" display="Ouvrir"/>
+    <hyperlink ref="K31" r:id="rId30" display="Ouvrir"/>
+    <hyperlink ref="K32" r:id="rId31" display="Ouvrir"/>
+    <hyperlink ref="K33" r:id="rId32" display="Ouvrir"/>
+    <hyperlink ref="K34" r:id="rId33" display="Ouvrir"/>
+    <hyperlink ref="K35" r:id="rId34" display="Ouvrir"/>
+    <hyperlink ref="K36" r:id="rId35" display="Ouvrir"/>
+    <hyperlink ref="K37" r:id="rId36" display="Ouvrir"/>
+    <hyperlink ref="K38" r:id="rId37" display="Ouvrir"/>
+    <hyperlink ref="K39" r:id="rId38" display="Ouvrir"/>
+    <hyperlink ref="K40" r:id="rId39" display="Ouvrir"/>
+    <hyperlink ref="K41" r:id="rId40" display="Ouvrir"/>
+    <hyperlink ref="K42" r:id="rId41" display="Ouvrir"/>
+    <hyperlink ref="K43" r:id="rId42" display="Ouvrir"/>
+    <hyperlink ref="K44" r:id="rId43" display="Ouvrir"/>
+    <hyperlink ref="K45" r:id="rId44" display="Ouvrir"/>
+    <hyperlink ref="K46" r:id="rId45" display="Ouvrir"/>
+    <hyperlink ref="K47" r:id="rId46" display="Ouvrir"/>
+    <hyperlink ref="K48" r:id="rId47" display="Ouvrir"/>
+    <hyperlink ref="K49" r:id="rId48" display="Ouvrir"/>
+    <hyperlink ref="K50" r:id="rId49" display="Ouvrir"/>
+    <hyperlink ref="K51" r:id="rId50" display="Ouvrir"/>
+    <hyperlink ref="K52" r:id="rId51" display="Ouvrir"/>
+    <hyperlink ref="K53" r:id="rId52" display="Ouvrir"/>
+  </hyperlinks>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+  <drawing r:id="rId53"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
   <dimension ref="A1:J28"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
@@ -15211,7 +18502,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="14" t="s">
-        <v>1103</v>
+        <v>1432</v>
       </c>
       <c r="B1" s="14" t="s">
         <v>40</v>
@@ -15220,7 +18511,7 @@
         <v>912</v>
       </c>
       <c r="D1" s="14" t="s">
-        <v>1104</v>
+        <v>1433</v>
       </c>
       <c r="E1" s="14" t="s">
         <v>915</v>
@@ -15232,84 +18523,84 @@
         <v>44</v>
       </c>
       <c r="H1" s="14" t="s">
-        <v>1105</v>
+        <v>1434</v>
       </c>
       <c r="I1" s="14" t="s">
-        <v>1106</v>
+        <v>1435</v>
       </c>
       <c r="J1" s="14" t="s">
-        <v>1107</v>
+        <v>1436</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="25" t="s">
-        <v>1108</v>
+        <v>1437</v>
       </c>
       <c r="B2" s="17" t="s">
         <v>939</v>
       </c>
       <c r="C2" s="17" t="s">
-        <v>1109</v>
+        <v>1438</v>
       </c>
       <c r="D2" s="17" t="s">
-        <v>1110</v>
+        <v>1439</v>
       </c>
       <c r="E2" s="17" t="s">
-        <v>1111</v>
+        <v>1440</v>
       </c>
       <c r="F2" s="17"/>
       <c r="G2" s="26" t="s">
-        <v>1112</v>
+        <v>1441</v>
       </c>
       <c r="H2" s="20" t="s">
-        <v>1113</v>
+        <v>1442</v>
       </c>
       <c r="I2" s="19" t="s">
-        <v>1114</v>
+        <v>1443</v>
       </c>
       <c r="J2" s="20"/>
     </row>
     <row r="3" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="25" t="s">
-        <v>1115</v>
+        <v>1444</v>
       </c>
       <c r="B3" s="17" t="s">
         <v>939</v>
       </c>
       <c r="C3" s="17" t="s">
-        <v>1116</v>
+        <v>1445</v>
       </c>
       <c r="D3" s="17" t="s">
-        <v>1117</v>
+        <v>1446</v>
       </c>
       <c r="E3" s="17" t="s">
-        <v>1118</v>
+        <v>1447</v>
       </c>
       <c r="F3" s="17"/>
       <c r="G3" s="26" t="s">
-        <v>1112</v>
+        <v>1441</v>
       </c>
       <c r="H3" s="20"/>
       <c r="I3" s="19"/>
       <c r="J3" s="20" t="s">
-        <v>1119</v>
+        <v>1448</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="25" t="s">
-        <v>1120</v>
+        <v>1449</v>
       </c>
       <c r="B4" s="17" t="s">
-        <v>1121</v>
+        <v>1450</v>
       </c>
       <c r="C4" s="17" t="s">
-        <v>1122</v>
+        <v>1451</v>
       </c>
       <c r="D4" s="17" t="s">
-        <v>1123</v>
+        <v>1452</v>
       </c>
       <c r="E4" s="17" t="s">
-        <v>1124</v>
+        <v>1453</v>
       </c>
       <c r="F4" s="18" t="s">
         <v>925</v>
@@ -15323,19 +18614,19 @@
     </row>
     <row r="5" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="25" t="s">
-        <v>1125</v>
+        <v>1454</v>
       </c>
       <c r="B5" s="17" t="s">
-        <v>1126</v>
+        <v>1455</v>
       </c>
       <c r="C5" s="17" t="s">
-        <v>1127</v>
+        <v>1456</v>
       </c>
       <c r="D5" s="17" t="s">
-        <v>1128</v>
+        <v>1457</v>
       </c>
       <c r="E5" s="17" t="s">
-        <v>1129</v>
+        <v>1458</v>
       </c>
       <c r="F5" s="17"/>
       <c r="G5" s="18" t="s">
@@ -15347,19 +18638,19 @@
     </row>
     <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="25" t="s">
-        <v>1130</v>
+        <v>1459</v>
       </c>
       <c r="B6" s="17" t="s">
-        <v>1131</v>
+        <v>1460</v>
       </c>
       <c r="C6" s="17" t="s">
-        <v>1122</v>
+        <v>1451</v>
       </c>
       <c r="D6" s="17" t="s">
-        <v>1132</v>
+        <v>1461</v>
       </c>
       <c r="E6" s="17" t="s">
-        <v>1133</v>
+        <v>1462</v>
       </c>
       <c r="F6" s="18" t="s">
         <v>925</v>
@@ -15373,19 +18664,19 @@
     </row>
     <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="25" t="s">
-        <v>1134</v>
+        <v>1463</v>
       </c>
       <c r="B7" s="17" t="s">
-        <v>1135</v>
+        <v>1464</v>
       </c>
       <c r="C7" s="17" t="s">
-        <v>1122</v>
+        <v>1451</v>
       </c>
       <c r="D7" s="17" t="s">
-        <v>1132</v>
+        <v>1461</v>
       </c>
       <c r="E7" s="17" t="s">
-        <v>1133</v>
+        <v>1462</v>
       </c>
       <c r="F7" s="18" t="s">
         <v>925</v>
@@ -15399,19 +18690,19 @@
     </row>
     <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="25" t="s">
-        <v>1136</v>
+        <v>1465</v>
       </c>
       <c r="B8" s="17" t="s">
-        <v>1137</v>
+        <v>1466</v>
       </c>
       <c r="C8" s="17" t="s">
-        <v>1122</v>
+        <v>1451</v>
       </c>
       <c r="D8" s="17" t="s">
-        <v>1138</v>
+        <v>1467</v>
       </c>
       <c r="E8" s="17" t="s">
-        <v>1133</v>
+        <v>1462</v>
       </c>
       <c r="F8" s="18" t="s">
         <v>925</v>
@@ -15425,19 +18716,19 @@
     </row>
     <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="25" t="s">
-        <v>1139</v>
+        <v>1468</v>
       </c>
       <c r="B9" s="17" t="s">
-        <v>1140</v>
+        <v>1469</v>
       </c>
       <c r="C9" s="17" t="s">
-        <v>1122</v>
+        <v>1451</v>
       </c>
       <c r="D9" s="17" t="s">
-        <v>1132</v>
+        <v>1461</v>
       </c>
       <c r="E9" s="17" t="s">
-        <v>1133</v>
+        <v>1462</v>
       </c>
       <c r="F9" s="18" t="s">
         <v>925</v>
@@ -15451,19 +18742,19 @@
     </row>
     <row r="10" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="25" t="s">
-        <v>1141</v>
+        <v>1470</v>
       </c>
       <c r="B10" s="17" t="s">
-        <v>1142</v>
+        <v>1471</v>
       </c>
       <c r="C10" s="17" t="s">
-        <v>1122</v>
+        <v>1451</v>
       </c>
       <c r="D10" s="17" t="s">
-        <v>1132</v>
+        <v>1461</v>
       </c>
       <c r="E10" s="17" t="s">
-        <v>1143</v>
+        <v>1472</v>
       </c>
       <c r="F10" s="18" t="s">
         <v>925</v>
@@ -15477,19 +18768,19 @@
     </row>
     <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="25" t="s">
-        <v>1144</v>
+        <v>1473</v>
       </c>
       <c r="B11" s="17" t="s">
-        <v>1145</v>
+        <v>1474</v>
       </c>
       <c r="C11" s="17" t="s">
-        <v>1122</v>
+        <v>1451</v>
       </c>
       <c r="D11" s="17" t="s">
-        <v>1132</v>
+        <v>1461</v>
       </c>
       <c r="E11" s="17" t="s">
-        <v>1133</v>
+        <v>1462</v>
       </c>
       <c r="F11" s="18" t="s">
         <v>925</v>
@@ -15503,19 +18794,19 @@
     </row>
     <row r="12" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="25" t="s">
-        <v>1146</v>
+        <v>1475</v>
       </c>
       <c r="B12" s="17" t="s">
-        <v>1147</v>
+        <v>1476</v>
       </c>
       <c r="C12" s="17" t="s">
-        <v>1122</v>
+        <v>1451</v>
       </c>
       <c r="D12" s="17" t="s">
-        <v>1132</v>
+        <v>1461</v>
       </c>
       <c r="E12" s="17" t="s">
-        <v>1148</v>
+        <v>1477</v>
       </c>
       <c r="F12" s="18" t="s">
         <v>925</v>
@@ -15529,19 +18820,19 @@
     </row>
     <row r="13" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="25" t="s">
-        <v>1149</v>
+        <v>1478</v>
       </c>
       <c r="B13" s="17" t="s">
-        <v>1150</v>
+        <v>1479</v>
       </c>
       <c r="C13" s="17" t="s">
-        <v>1122</v>
+        <v>1451</v>
       </c>
       <c r="D13" s="17" t="s">
-        <v>1132</v>
+        <v>1461</v>
       </c>
       <c r="E13" s="17" t="s">
-        <v>1151</v>
+        <v>1480</v>
       </c>
       <c r="F13" s="18" t="s">
         <v>925</v>
@@ -15555,19 +18846,19 @@
     </row>
     <row r="14" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="25" t="s">
-        <v>1152</v>
+        <v>1481</v>
       </c>
       <c r="B14" s="17" t="s">
-        <v>1153</v>
+        <v>1482</v>
       </c>
       <c r="C14" s="17" t="s">
-        <v>1122</v>
+        <v>1451</v>
       </c>
       <c r="D14" s="17" t="s">
-        <v>1132</v>
+        <v>1461</v>
       </c>
       <c r="E14" s="17" t="s">
-        <v>1133</v>
+        <v>1462</v>
       </c>
       <c r="F14" s="18" t="s">
         <v>925</v>
@@ -15581,19 +18872,19 @@
     </row>
     <row r="15" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="25" t="s">
-        <v>1154</v>
+        <v>1483</v>
       </c>
       <c r="B15" s="17" t="s">
-        <v>1155</v>
+        <v>1484</v>
       </c>
       <c r="C15" s="17" t="s">
-        <v>1122</v>
+        <v>1451</v>
       </c>
       <c r="D15" s="17" t="s">
-        <v>1132</v>
+        <v>1461</v>
       </c>
       <c r="E15" s="17" t="s">
-        <v>1133</v>
+        <v>1462</v>
       </c>
       <c r="F15" s="18" t="s">
         <v>925</v>
@@ -15607,19 +18898,19 @@
     </row>
     <row r="16" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="25" t="s">
-        <v>1156</v>
+        <v>1485</v>
       </c>
       <c r="B16" s="17" t="s">
-        <v>1157</v>
+        <v>1486</v>
       </c>
       <c r="C16" s="17" t="s">
-        <v>1122</v>
+        <v>1451</v>
       </c>
       <c r="D16" s="17" t="s">
-        <v>1132</v>
+        <v>1461</v>
       </c>
       <c r="E16" s="17" t="s">
-        <v>1133</v>
+        <v>1462</v>
       </c>
       <c r="F16" s="18" t="s">
         <v>925</v>
@@ -15633,19 +18924,19 @@
     </row>
     <row r="17" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="25" t="s">
-        <v>1158</v>
+        <v>1487</v>
       </c>
       <c r="B17" s="17" t="s">
-        <v>1159</v>
+        <v>1488</v>
       </c>
       <c r="C17" s="17" t="s">
-        <v>1122</v>
+        <v>1451</v>
       </c>
       <c r="D17" s="17" t="s">
-        <v>1132</v>
+        <v>1461</v>
       </c>
       <c r="E17" s="17" t="s">
-        <v>1133</v>
+        <v>1462</v>
       </c>
       <c r="F17" s="18" t="s">
         <v>925</v>
@@ -15659,19 +18950,19 @@
     </row>
     <row r="18" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="25" t="s">
-        <v>1160</v>
+        <v>1489</v>
       </c>
       <c r="B18" s="17" t="s">
-        <v>1161</v>
+        <v>1490</v>
       </c>
       <c r="C18" s="17" t="s">
-        <v>1122</v>
+        <v>1451</v>
       </c>
       <c r="D18" s="17" t="s">
-        <v>1132</v>
+        <v>1461</v>
       </c>
       <c r="E18" s="17" t="s">
-        <v>1133</v>
+        <v>1462</v>
       </c>
       <c r="F18" s="18" t="s">
         <v>925</v>
@@ -15685,19 +18976,19 @@
     </row>
     <row r="19" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="25" t="s">
-        <v>1162</v>
+        <v>1491</v>
       </c>
       <c r="B19" s="17" t="s">
-        <v>1163</v>
+        <v>1492</v>
       </c>
       <c r="C19" s="17" t="s">
-        <v>1122</v>
+        <v>1451</v>
       </c>
       <c r="D19" s="17" t="s">
-        <v>1132</v>
+        <v>1461</v>
       </c>
       <c r="E19" s="17" t="s">
-        <v>1164</v>
+        <v>1493</v>
       </c>
       <c r="F19" s="18" t="s">
         <v>925</v>
@@ -15711,19 +19002,19 @@
     </row>
     <row r="20" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="25" t="s">
-        <v>1165</v>
+        <v>1494</v>
       </c>
       <c r="B20" s="17" t="s">
-        <v>1166</v>
+        <v>1495</v>
       </c>
       <c r="C20" s="17" t="s">
-        <v>1122</v>
+        <v>1451</v>
       </c>
       <c r="D20" s="17" t="s">
-        <v>1132</v>
+        <v>1461</v>
       </c>
       <c r="E20" s="17" t="s">
-        <v>1164</v>
+        <v>1493</v>
       </c>
       <c r="F20" s="18" t="s">
         <v>925</v>
@@ -15737,19 +19028,19 @@
     </row>
     <row r="21" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="25" t="s">
-        <v>1167</v>
+        <v>1496</v>
       </c>
       <c r="B21" s="17" t="s">
-        <v>1168</v>
+        <v>1497</v>
       </c>
       <c r="C21" s="17" t="s">
-        <v>1122</v>
+        <v>1451</v>
       </c>
       <c r="D21" s="17" t="s">
-        <v>1169</v>
+        <v>1498</v>
       </c>
       <c r="E21" s="17" t="s">
-        <v>1170</v>
+        <v>1499</v>
       </c>
       <c r="F21" s="18" t="s">
         <v>925</v>
@@ -15763,19 +19054,19 @@
     </row>
     <row r="22" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="25" t="s">
-        <v>1171</v>
+        <v>1500</v>
       </c>
       <c r="B22" s="17" t="s">
-        <v>1172</v>
+        <v>1501</v>
       </c>
       <c r="C22" s="17" t="s">
-        <v>1122</v>
+        <v>1451</v>
       </c>
       <c r="D22" s="17" t="s">
-        <v>1132</v>
+        <v>1461</v>
       </c>
       <c r="E22" s="17" t="s">
-        <v>1173</v>
+        <v>1502</v>
       </c>
       <c r="F22" s="18" t="s">
         <v>925</v>
@@ -15789,19 +19080,19 @@
     </row>
     <row r="23" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="25" t="s">
-        <v>1174</v>
+        <v>1503</v>
       </c>
       <c r="B23" s="17" t="s">
-        <v>1175</v>
+        <v>1504</v>
       </c>
       <c r="C23" s="17" t="s">
-        <v>1116</v>
+        <v>1445</v>
       </c>
       <c r="D23" s="17" t="s">
-        <v>1176</v>
+        <v>1505</v>
       </c>
       <c r="E23" s="17" t="s">
-        <v>1177</v>
+        <v>1506</v>
       </c>
       <c r="F23" s="18" t="s">
         <v>925</v>
@@ -15815,7 +19106,7 @@
     </row>
     <row r="25" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="2" t="s">
-        <v>1178</v>
+        <v>1507</v>
       </c>
       <c r="B25" s="2"/>
       <c r="C25" s="2"/>
@@ -15825,7 +19116,7 @@
     </row>
     <row r="26" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="2" t="s">
-        <v>1179</v>
+        <v>1508</v>
       </c>
       <c r="B26" s="2"/>
       <c r="C26" s="2"/>
@@ -15835,7 +19126,7 @@
     </row>
     <row r="27" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="2" t="s">
-        <v>1180</v>
+        <v>1509</v>
       </c>
       <c r="B27" s="2"/>
       <c r="C27" s="2"/>
@@ -15845,7 +19136,7 @@
     </row>
     <row r="28" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="2" t="s">
-        <v>1181</v>
+        <v>1510</v>
       </c>
       <c r="B28" s="2"/>
       <c r="C28" s="2"/>
@@ -15917,12 +19208,12 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:E22"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="30"/>
@@ -15936,10 +19227,10 @@
         <v>911</v>
       </c>
       <c r="B1" s="14" t="s">
-        <v>1182</v>
+        <v>1511</v>
       </c>
       <c r="C1" s="14" t="s">
-        <v>1183</v>
+        <v>1512</v>
       </c>
       <c r="D1" s="14" t="s">
         <v>915</v>
@@ -15950,16 +19241,16 @@
     </row>
     <row r="2" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="25" t="s">
-        <v>1184</v>
+        <v>1513</v>
       </c>
       <c r="B2" s="17" t="s">
-        <v>1185</v>
+        <v>1514</v>
       </c>
       <c r="C2" s="17" t="s">
-        <v>1186</v>
+        <v>1515</v>
       </c>
       <c r="D2" s="17" t="s">
-        <v>1187</v>
+        <v>1516</v>
       </c>
       <c r="E2" s="27" t="s">
         <v>925</v>
@@ -15967,16 +19258,16 @@
     </row>
     <row r="3" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="25" t="s">
-        <v>1188</v>
+        <v>1517</v>
       </c>
       <c r="B3" s="17" t="s">
-        <v>1189</v>
+        <v>1518</v>
       </c>
       <c r="C3" s="17" t="s">
         <v>315</v>
       </c>
       <c r="D3" s="17" t="s">
-        <v>1190</v>
+        <v>1519</v>
       </c>
       <c r="E3" s="27" t="s">
         <v>925</v>
@@ -15984,16 +19275,16 @@
     </row>
     <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="25" t="s">
-        <v>1191</v>
+        <v>1520</v>
       </c>
       <c r="B4" s="17" t="s">
-        <v>1192</v>
+        <v>1521</v>
       </c>
       <c r="C4" s="17" t="s">
-        <v>1193</v>
+        <v>1522</v>
       </c>
       <c r="D4" s="17" t="s">
-        <v>1194</v>
+        <v>1523</v>
       </c>
       <c r="E4" s="27" t="s">
         <v>925</v>
@@ -16001,16 +19292,16 @@
     </row>
     <row r="5" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="25" t="s">
-        <v>1195</v>
+        <v>1524</v>
       </c>
       <c r="B5" s="17" t="s">
-        <v>1196</v>
+        <v>1525</v>
       </c>
       <c r="C5" s="17" t="s">
-        <v>1197</v>
+        <v>1526</v>
       </c>
       <c r="D5" s="17" t="s">
-        <v>1198</v>
+        <v>1527</v>
       </c>
       <c r="E5" s="27" t="s">
         <v>925</v>
@@ -16018,16 +19309,16 @@
     </row>
     <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="25" t="s">
-        <v>1199</v>
+        <v>1528</v>
       </c>
       <c r="B6" s="17" t="s">
-        <v>1200</v>
+        <v>1529</v>
       </c>
       <c r="C6" s="17" t="s">
-        <v>1201</v>
+        <v>1530</v>
       </c>
       <c r="D6" s="17" t="s">
-        <v>1202</v>
+        <v>1531</v>
       </c>
       <c r="E6" s="27" t="s">
         <v>925</v>
@@ -16035,16 +19326,16 @@
     </row>
     <row r="7" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="25" t="s">
-        <v>1203</v>
+        <v>1532</v>
       </c>
       <c r="B7" s="17" t="s">
-        <v>1204</v>
+        <v>1533</v>
       </c>
       <c r="C7" s="17" t="s">
-        <v>1205</v>
+        <v>1534</v>
       </c>
       <c r="D7" s="17" t="s">
-        <v>1206</v>
+        <v>1535</v>
       </c>
       <c r="E7" s="27" t="s">
         <v>925</v>
@@ -16052,16 +19343,16 @@
     </row>
     <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="25" t="s">
-        <v>1207</v>
+        <v>1536</v>
       </c>
       <c r="B8" s="17" t="s">
-        <v>1208</v>
+        <v>1537</v>
       </c>
       <c r="C8" s="17" t="s">
-        <v>1209</v>
+        <v>1538</v>
       </c>
       <c r="D8" s="17" t="s">
-        <v>1210</v>
+        <v>1539</v>
       </c>
       <c r="E8" s="27" t="s">
         <v>925</v>
@@ -16069,16 +19360,16 @@
     </row>
     <row r="9" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="25" t="s">
-        <v>1211</v>
+        <v>1540</v>
       </c>
       <c r="B9" s="17" t="s">
-        <v>1212</v>
+        <v>1541</v>
       </c>
       <c r="C9" s="17" t="s">
-        <v>1213</v>
+        <v>1542</v>
       </c>
       <c r="D9" s="17" t="s">
-        <v>1214</v>
+        <v>1543</v>
       </c>
       <c r="E9" s="27" t="s">
         <v>925</v>
@@ -16086,16 +19377,16 @@
     </row>
     <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="25" t="s">
-        <v>1215</v>
+        <v>1544</v>
       </c>
       <c r="B10" s="17" t="s">
-        <v>1216</v>
+        <v>1545</v>
       </c>
       <c r="C10" s="17" t="s">
         <v>50</v>
       </c>
       <c r="D10" s="17" t="s">
-        <v>1217</v>
+        <v>1546</v>
       </c>
       <c r="E10" s="27" t="s">
         <v>925</v>
@@ -16103,16 +19394,16 @@
     </row>
     <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="25" t="s">
-        <v>1218</v>
+        <v>1547</v>
       </c>
       <c r="B11" s="17" t="s">
-        <v>1219</v>
+        <v>1548</v>
       </c>
       <c r="C11" s="17" t="s">
-        <v>1220</v>
+        <v>1549</v>
       </c>
       <c r="D11" s="17" t="s">
-        <v>1221</v>
+        <v>1550</v>
       </c>
       <c r="E11" s="27" t="s">
         <v>925</v>
@@ -16120,16 +19411,16 @@
     </row>
     <row r="12" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="25" t="s">
-        <v>1222</v>
+        <v>1551</v>
       </c>
       <c r="B12" s="17" t="s">
-        <v>1223</v>
+        <v>1552</v>
       </c>
       <c r="C12" s="17" t="s">
-        <v>1224</v>
+        <v>1553</v>
       </c>
       <c r="D12" s="17" t="s">
-        <v>1225</v>
+        <v>1554</v>
       </c>
       <c r="E12" s="27" t="s">
         <v>925</v>
@@ -16137,16 +19428,16 @@
     </row>
     <row r="13" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="25" t="s">
-        <v>1226</v>
+        <v>1555</v>
       </c>
       <c r="B13" s="17" t="s">
-        <v>1227</v>
+        <v>1556</v>
       </c>
       <c r="C13" s="17" t="s">
-        <v>1228</v>
+        <v>1557</v>
       </c>
       <c r="D13" s="17" t="s">
-        <v>1229</v>
+        <v>1558</v>
       </c>
       <c r="E13" s="27" t="s">
         <v>925</v>
@@ -16154,16 +19445,16 @@
     </row>
     <row r="14" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="25" t="s">
-        <v>1230</v>
+        <v>1559</v>
       </c>
       <c r="B14" s="17" t="s">
-        <v>1231</v>
+        <v>1560</v>
       </c>
       <c r="C14" s="17" t="s">
-        <v>1232</v>
+        <v>1561</v>
       </c>
       <c r="D14" s="17" t="s">
-        <v>1233</v>
+        <v>1562</v>
       </c>
       <c r="E14" s="27" t="s">
         <v>925</v>
@@ -16171,33 +19462,33 @@
     </row>
     <row r="15" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="25" t="s">
-        <v>1234</v>
+        <v>1563</v>
       </c>
       <c r="B15" s="17" t="s">
-        <v>1235</v>
+        <v>1564</v>
       </c>
       <c r="C15" s="17" t="s">
-        <v>1236</v>
+        <v>1565</v>
       </c>
       <c r="D15" s="17" t="s">
-        <v>1237</v>
+        <v>1566</v>
       </c>
       <c r="E15" s="27" t="s">
         <v>925</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="16" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="25" t="s">
-        <v>1238</v>
+        <v>1567</v>
       </c>
       <c r="B16" s="17" t="s">
-        <v>1239</v>
+        <v>1568</v>
       </c>
       <c r="C16" s="17" t="s">
-        <v>1240</v>
+        <v>1569</v>
       </c>
       <c r="D16" s="17" t="s">
-        <v>1241</v>
+        <v>1570</v>
       </c>
       <c r="E16" s="27" t="s">
         <v>925</v>
@@ -16205,18 +19496,103 @@
     </row>
     <row r="17" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="25" t="s">
-        <v>1242</v>
+        <v>1571</v>
       </c>
       <c r="B17" s="17" t="s">
-        <v>1243</v>
+        <v>1572</v>
       </c>
       <c r="C17" s="17" t="s">
-        <v>1244</v>
+        <v>1573</v>
       </c>
       <c r="D17" s="17" t="s">
-        <v>1245</v>
-      </c>
-      <c r="E17" s="28"/>
+        <v>1574</v>
+      </c>
+      <c r="E17" s="27" t="s">
+        <v>925</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="25" t="s">
+        <v>1139</v>
+      </c>
+      <c r="B18" s="17" t="s">
+        <v>1575</v>
+      </c>
+      <c r="C18" s="17" t="s">
+        <v>1576</v>
+      </c>
+      <c r="D18" s="17" t="s">
+        <v>1577</v>
+      </c>
+      <c r="E18" s="27" t="s">
+        <v>925</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="25" t="s">
+        <v>1578</v>
+      </c>
+      <c r="B19" s="17" t="s">
+        <v>1579</v>
+      </c>
+      <c r="C19" s="17" t="s">
+        <v>1580</v>
+      </c>
+      <c r="D19" s="17" t="s">
+        <v>1581</v>
+      </c>
+      <c r="E19" s="27" t="s">
+        <v>925</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="25" t="s">
+        <v>1157</v>
+      </c>
+      <c r="B20" s="17" t="s">
+        <v>1582</v>
+      </c>
+      <c r="C20" s="17" t="s">
+        <v>1583</v>
+      </c>
+      <c r="D20" s="17" t="s">
+        <v>1584</v>
+      </c>
+      <c r="E20" s="27" t="s">
+        <v>925</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="25" t="s">
+        <v>1585</v>
+      </c>
+      <c r="B21" s="17" t="s">
+        <v>1586</v>
+      </c>
+      <c r="C21" s="17" t="s">
+        <v>1587</v>
+      </c>
+      <c r="D21" s="17" t="s">
+        <v>1588</v>
+      </c>
+      <c r="E21" s="27" t="s">
+        <v>925</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="25" t="s">
+        <v>1589</v>
+      </c>
+      <c r="B22" s="17" t="s">
+        <v>1590</v>
+      </c>
+      <c r="C22" s="17" t="s">
+        <v>1591</v>
+      </c>
+      <c r="D22" s="17" t="s">
+        <v>1592</v>
+      </c>
+      <c r="E22" s="28"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -16235,6 +19611,11 @@
     <hyperlink ref="E14" r:id="rId13" display="Ouvrir"/>
     <hyperlink ref="E15" r:id="rId14" display="Ouvrir"/>
     <hyperlink ref="E16" r:id="rId15" display="Ouvrir"/>
+    <hyperlink ref="E17" r:id="rId16" display="Ouvrir"/>
+    <hyperlink ref="E18" r:id="rId17" display="Ouvrir"/>
+    <hyperlink ref="E19" r:id="rId18" display="Ouvrir"/>
+    <hyperlink ref="E20" r:id="rId19" display="Ouvrir"/>
+    <hyperlink ref="E21" r:id="rId20" display="Ouvrir"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -16246,7 +19627,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
@@ -16261,10 +19642,10 @@
   <sheetData>
     <row r="1" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="14" t="s">
-        <v>1246</v>
+        <v>1593</v>
       </c>
       <c r="B1" s="14" t="s">
-        <v>1247</v>
+        <v>1594</v>
       </c>
       <c r="C1" s="14" t="s">
         <v>44</v>
@@ -16272,10 +19653,10 @@
     </row>
     <row r="2" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="25" t="s">
-        <v>1248</v>
+        <v>1595</v>
       </c>
       <c r="B2" s="17" t="s">
-        <v>1249</v>
+        <v>1596</v>
       </c>
       <c r="C2" s="27" t="s">
         <v>925</v>
@@ -16283,10 +19664,10 @@
     </row>
     <row r="3" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="25" t="s">
-        <v>1250</v>
+        <v>1597</v>
       </c>
       <c r="B3" s="17" t="s">
-        <v>1251</v>
+        <v>1598</v>
       </c>
       <c r="C3" s="27" t="s">
         <v>925</v>
@@ -16294,10 +19675,10 @@
     </row>
     <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="25" t="s">
-        <v>1252</v>
+        <v>1599</v>
       </c>
       <c r="B4" s="17" t="s">
-        <v>1253</v>
+        <v>1600</v>
       </c>
       <c r="C4" s="27" t="s">
         <v>925</v>
@@ -16305,10 +19686,10 @@
     </row>
     <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="25" t="s">
-        <v>1254</v>
+        <v>1601</v>
       </c>
       <c r="B5" s="17" t="s">
-        <v>1255</v>
+        <v>1602</v>
       </c>
       <c r="C5" s="27" t="s">
         <v>925</v>
@@ -16316,10 +19697,10 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="25" t="s">
-        <v>1256</v>
+        <v>1603</v>
       </c>
       <c r="B6" s="17" t="s">
-        <v>1257</v>
+        <v>1604</v>
       </c>
       <c r="C6" s="27" t="s">
         <v>925</v>
@@ -16327,10 +19708,10 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="25" t="s">
-        <v>1258</v>
+        <v>1605</v>
       </c>
       <c r="B7" s="17" t="s">
-        <v>1259</v>
+        <v>1606</v>
       </c>
       <c r="C7" s="27" t="s">
         <v>925</v>
@@ -16338,10 +19719,10 @@
     </row>
     <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="25" t="s">
-        <v>1260</v>
+        <v>1607</v>
       </c>
       <c r="B8" s="17" t="s">
-        <v>1261</v>
+        <v>1608</v>
       </c>
       <c r="C8" s="27" t="s">
         <v>925</v>
@@ -16349,10 +19730,10 @@
     </row>
     <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="25" t="s">
-        <v>1262</v>
+        <v>1609</v>
       </c>
       <c r="B9" s="17" t="s">
-        <v>1263</v>
+        <v>1610</v>
       </c>
       <c r="C9" s="27" t="s">
         <v>925</v>
@@ -16360,10 +19741,10 @@
     </row>
     <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="25" t="s">
-        <v>1264</v>
+        <v>1611</v>
       </c>
       <c r="B10" s="17" t="s">
-        <v>1265</v>
+        <v>1612</v>
       </c>
       <c r="C10" s="27" t="s">
         <v>925</v>
@@ -16371,10 +19752,10 @@
     </row>
     <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="25" t="s">
-        <v>1266</v>
+        <v>1613</v>
       </c>
       <c r="B11" s="17" t="s">
-        <v>1267</v>
+        <v>1614</v>
       </c>
       <c r="C11" s="27" t="s">
         <v>925</v>
@@ -16382,7 +19763,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="10" t="s">
-        <v>1268</v>
+        <v>1615</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Final check fixes: pro-group verification, outdoor qualifiers, legal-notice link
- facebook-instagram.md: verify a group is private and pro-only (and what
  price the existing LES PRO DU BÂTIMENT post shows) before any trade
  price; ad D now "selon finition et pose" (141 characters).
- kit-de-vente.md: Leboncoin uses line qualified for every outdoor use.
- index.html: footer links to the store's legal notice.
- README: legal notice must also cover the landing page's host.
- prospects-minyala.xlsx: every outdoor Leboncoin listing carries the
  qualifier; group rows say to check pro-only membership first.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Xqm9tFtdvLdJdkiWw2VVp6
</commit_message>
<xml_diff>
--- a/minyala/prospects-minyala.xlsx
+++ b/minyala/prospects-minyala.xlsx
@@ -2849,7 +2849,7 @@
     <t xml:space="preserve">Annonce localisée à Gennevilliers, et une 2e à Vernon (27) dès que l'adresse est connue</t>
   </si>
   <si>
-    <t xml:space="preserve">Ouvrir un compte Pro (obligatoire pour une entreprise). Une annonce par usage : terrasse, abords de piscine (selon finition et pose, à écrire dans le titre et le texte), sol intérieur. Prix au m², minimum 25 m², retrait sur rendez-vous. Republier au printemps.</t>
+    <t xml:space="preserve">Ouvrir un compte Pro (obligatoire pour une entreprise). Une annonce par usage : terrasse, abords de piscine, sol intérieur — pour chaque annonce extérieure (terrasse, piscine), écrire « selon finition et pose » dans le titre et le texte. Prix au m², minimum 25 m², retrait sur rendez-vous. Republier au printemps.</t>
   </si>
   <si>
     <t xml:space="preserve">Compte Pro gratuit ; 50 annonces offertes en Maison &amp; Jardin, puis payant (à vérifier)</t>
@@ -4427,7 +4427,7 @@
     <t xml:space="preserve">Non relevé</t>
   </si>
   <si>
-    <t xml:space="preserve">Annonce déjà présente (doublon évité le 12/10/2026) : ne pas republier, répondre aux commentaires et messages. Lien du groupe à ajouter.</t>
+    <t xml:space="preserve">Annonce déjà présente (doublon évité le 12/10/2026). Vérifier : groupe privé et réservé aux pros ? Quel prix affiche l'annonce ? Si le groupe est ouvert aux particuliers, modifier l'annonce au prix public 35 €/m² pierre seule + « Pros : tarif sur demande ». Sinon, répondre seulement. Lien du groupe à ajouter.</t>
   </si>
   <si>
     <t xml:space="preserve">avant le 12/10/2026</t>
@@ -4607,7 +4607,7 @@
     <t xml:space="preserve">~5 400, privé (2023)</t>
   </si>
   <si>
-    <t xml:space="preserve">Se présenter comme fournisseur aux carreleurs, maçons et paysagistes. Pas de démarchage en message privé.</t>
+    <t xml:space="preserve">Groupe privé (~5 400, 2023). Vérifier qu'il est réservé aux pros avant d'y publier le prix pro. Se présenter comme fournisseur ; pas de démarchage en message privé.</t>
   </si>
   <si>
     <t xml:space="preserve">• Liens et effectifs viennent d'articles de presse (2016–2024) : vérifiez que chaque groupe existe toujours, son nom exact et son règlement une fois connecté.</t>
@@ -19789,7 +19789,7 @@
       </c>
       <c r="J2" s="20"/>
     </row>
-    <row r="3" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="25" t="s">
         <v>1446</v>
       </c>
@@ -20307,7 +20307,7 @@
       <c r="I22" s="19"/>
       <c r="J22" s="20"/>
     </row>
-    <row r="23" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="23" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="25" t="s">
         <v>1506</v>
       </c>

</xml_diff>

<commit_message>
ChatGPT channel verdict (US-only), IFZA note for the accountant
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Xqm9tFtdvLdJdkiWw2VVp6
</commit_message>
<xml_diff>
--- a/minyala/prospects-minyala.xlsx
+++ b/minyala/prospects-minyala.xlsx
@@ -4853,10 +4853,10 @@
     <t xml:space="preserve">Acheteurs qui demandent conseil à ChatGPT</t>
   </si>
   <si>
-    <t xml:space="preserve">Disponibilité en France à vérifier</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Shopify admin &gt; Paramètres &gt; Canaux de vente &gt; Agentic storefronts. Masquer d'abord les produits « Acompte ».</t>
+    <t xml:space="preserve">Non disponible (13/10/2026) : réservé aux boutiques qui vendent aux États-Unis</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pas de canal de vente possible pour l'instant. Visibilité gratuite : les pages du site peuvent être citées par la recherche de ChatGPT. D'ici là : passer les produits « Acompte » en « Non répertorié », remplir les CGV et la politique de remboursement, ajouter des photos réelles.</t>
   </si>
   <si>
     <t xml:space="preserve">E-mail / téléphone aux pros</t>
@@ -20794,7 +20794,7 @@
         <v>925</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="21" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="25" t="s">
         <v>1589</v>
       </c>

</xml_diff>